<commit_message>
Chunk data review: drop repeated examples, fix six label-as-mistake cards
An audit of all 1,430 cards found 632 whose drafted example 2 or 3 repeated
example 1, and 6 whose workbook "wrong version" cell held a label ("Future
plan") rather than a mistake. Repeats are dropped at merge time; those six
use the drafted mistake with the label kept as the tip. Review workbooks
rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XivsNLnRJbP4wB6VLVY5B5
</commit_message>
<xml_diff>
--- a/content/chunk-library/Grammar_Library_Review.xlsx
+++ b/content/chunk-library/Grammar_Library_Review.xlsx
@@ -1115,13 +1115,21 @@
           <t>Main apne chacha se milne jaane wala hoon.</t>
         </is>
       </c>
-      <c r="Y3" s="13" t="inlineStr">
-        <is>
-          <t>Future plan</t>
-        </is>
-      </c>
-      <c r="Z3" s="13" t="inlineStr"/>
-      <c r="AA3" s="13" t="inlineStr"/>
+      <c r="Y3" s="14" t="inlineStr">
+        <is>
+          <t>I'm going to went.</t>
+        </is>
+      </c>
+      <c r="Z3" s="14" t="inlineStr">
+        <is>
+          <t>I'm going to go.</t>
+        </is>
+      </c>
+      <c r="AA3" s="14" t="inlineStr">
+        <is>
+          <t>After "going to" use the base verb.</t>
+        </is>
+      </c>
       <c r="AB3" s="14" t="inlineStr">
         <is>
           <t>I'm going to + base verb.</t>
@@ -3833,11 +3841,7 @@
           <t>Will you come tomorrow?</t>
         </is>
       </c>
-      <c r="W16" s="14" t="inlineStr">
-        <is>
-          <t>Will you help me?</t>
-        </is>
-      </c>
+      <c r="W16" s="13" t="inlineStr"/>
       <c r="X16" s="13" t="inlineStr">
         <is>
           <t>Kya tum meri madad karoge?</t>
@@ -4686,14 +4690,10 @@
       </c>
       <c r="V20" s="14" t="inlineStr">
         <is>
-          <t>May I come in?</t>
-        </is>
-      </c>
-      <c r="W20" s="14" t="inlineStr">
-        <is>
           <t>Can I sit here?</t>
         </is>
       </c>
+      <c r="W20" s="13" t="inlineStr"/>
       <c r="X20" s="13" t="inlineStr">
         <is>
           <t>Kya main andar aa sakta hoon?</t>
@@ -5542,14 +5542,10 @@
       </c>
       <c r="V24" s="14" t="inlineStr">
         <is>
-          <t>What do you call "chammach" in English?</t>
-        </is>
-      </c>
-      <c r="W24" s="14" t="inlineStr">
-        <is>
           <t>What do you call this in English?</t>
         </is>
       </c>
+      <c r="W24" s="13" t="inlineStr"/>
       <c r="X24" s="13" t="inlineStr">
         <is>
           <t>Chammach ko English mein kya kehte hain?</t>
@@ -7241,11 +7237,7 @@
           <t>I don't want to eat.</t>
         </is>
       </c>
-      <c r="W32" s="14" t="inlineStr">
-        <is>
-          <t>I don't want to go out today.</t>
-        </is>
-      </c>
+      <c r="W32" s="13" t="inlineStr"/>
       <c r="X32" s="13" t="inlineStr">
         <is>
           <t>Main aaj bahar nahi jaana chahta.</t>
@@ -7670,14 +7662,10 @@
       </c>
       <c r="V34" s="14" t="inlineStr">
         <is>
-          <t>My hobby is painting.</t>
-        </is>
-      </c>
-      <c r="W34" s="14" t="inlineStr">
-        <is>
           <t>My hobbies are reading and cooking.</t>
         </is>
       </c>
+      <c r="W34" s="13" t="inlineStr"/>
       <c r="X34" s="13" t="inlineStr">
         <is>
           <t>Mera shauk painting karna hai.</t>
@@ -7878,14 +7866,10 @@
       </c>
       <c r="V35" s="14" t="inlineStr">
         <is>
-          <t>What's your name?</t>
-        </is>
-      </c>
-      <c r="W35" s="14" t="inlineStr">
-        <is>
           <t>What's your number?</t>
         </is>
       </c>
+      <c r="W35" s="13" t="inlineStr"/>
       <c r="X35" s="13" t="inlineStr">
         <is>
           <t>Tumhara naam kya hai?</t>
@@ -8298,14 +8282,10 @@
       </c>
       <c r="V37" s="14" t="inlineStr">
         <is>
-          <t>Which colour do you like?</t>
-        </is>
-      </c>
-      <c r="W37" s="14" t="inlineStr">
-        <is>
           <t>Which one do you like?</t>
         </is>
       </c>
+      <c r="W37" s="13" t="inlineStr"/>
       <c r="X37" s="13" t="inlineStr">
         <is>
           <t>Tumhe kaunsa rang pasand hai?</t>
@@ -8717,11 +8697,7 @@
           <t>How many brothers do you have?</t>
         </is>
       </c>
-      <c r="W39" s="14" t="inlineStr">
-        <is>
-          <t>How many books do you have?</t>
-        </is>
-      </c>
+      <c r="W39" s="13" t="inlineStr"/>
       <c r="X39" s="13" t="inlineStr">
         <is>
           <t>Tumhare paas kitni kitaabein hain?</t>
@@ -9346,14 +9322,10 @@
       </c>
       <c r="V42" s="14" t="inlineStr">
         <is>
-          <t>What did you do yesterday?</t>
-        </is>
-      </c>
-      <c r="W42" s="14" t="inlineStr">
-        <is>
           <t>What did you do on the weekend?</t>
         </is>
       </c>
+      <c r="W42" s="13" t="inlineStr"/>
       <c r="X42" s="13" t="inlineStr">
         <is>
           <t>Tumne kal kya kiya?</t>
@@ -9554,14 +9526,10 @@
       </c>
       <c r="V43" s="14" t="inlineStr">
         <is>
-          <t>Where do you live?</t>
-        </is>
-      </c>
-      <c r="W43" s="14" t="inlineStr">
-        <is>
           <t>Where do you work?</t>
         </is>
       </c>
+      <c r="W43" s="13" t="inlineStr"/>
       <c r="X43" s="13" t="inlineStr">
         <is>
           <t>Tum kahan rehte ho?</t>
@@ -9978,14 +9946,10 @@
       </c>
       <c r="V45" s="14" t="inlineStr">
         <is>
-          <t>Do you have a pen?</t>
-        </is>
-      </c>
-      <c r="W45" s="14" t="inlineStr">
-        <is>
           <t>Do you have change?</t>
         </is>
       </c>
+      <c r="W45" s="13" t="inlineStr"/>
       <c r="X45" s="13" t="inlineStr">
         <is>
           <t>Kya tumhare paas pen hai?</t>
@@ -11047,13 +11011,21 @@
           <t>Maine kabhi sushi nahi khaya.</t>
         </is>
       </c>
-      <c r="Y50" s="13" t="inlineStr">
-        <is>
-          <t>Present perfect (experience)</t>
-        </is>
-      </c>
-      <c r="Z50" s="13" t="inlineStr"/>
-      <c r="AA50" s="13" t="inlineStr"/>
+      <c r="Y50" s="14" t="inlineStr">
+        <is>
+          <t>I have never went.</t>
+        </is>
+      </c>
+      <c r="Z50" s="14" t="inlineStr">
+        <is>
+          <t>I have never been.</t>
+        </is>
+      </c>
+      <c r="AA50" s="14" t="inlineStr">
+        <is>
+          <t>Use the past participle.</t>
+        </is>
+      </c>
       <c r="AB50" s="14" t="inlineStr">
         <is>
           <t>I have never + past participle.</t>
@@ -12742,14 +12714,10 @@
       </c>
       <c r="V58" s="14" t="inlineStr">
         <is>
-          <t>I'm about to leave.</t>
-        </is>
-      </c>
-      <c r="W58" s="14" t="inlineStr">
-        <is>
           <t>The film is about to start.</t>
         </is>
       </c>
+      <c r="W58" s="13" t="inlineStr"/>
       <c r="X58" s="13" t="inlineStr">
         <is>
           <t>Main nikalne wala hoon.</t>
@@ -13601,11 +13569,7 @@
           <t>You should rest.</t>
         </is>
       </c>
-      <c r="W62" s="14" t="inlineStr">
-        <is>
-          <t>You should see a doctor.</t>
-        </is>
-      </c>
+      <c r="W62" s="13" t="inlineStr"/>
       <c r="X62" s="13" t="inlineStr">
         <is>
           <t>Tumhe doctor ko dikhana chahiye.</t>
@@ -14642,14 +14606,10 @@
       </c>
       <c r="V67" s="14" t="inlineStr">
         <is>
-          <t>This is the best phone.</t>
-        </is>
-      </c>
-      <c r="W67" s="14" t="inlineStr">
-        <is>
           <t>She's the tallest in class.</t>
         </is>
       </c>
+      <c r="W67" s="13" t="inlineStr"/>
       <c r="X67" s="13" t="inlineStr">
         <is>
           <t>Yeh sabse achha phone hai.</t>
@@ -15065,11 +15025,7 @@
           <t>Either tea or coffee.</t>
         </is>
       </c>
-      <c r="W69" s="14" t="inlineStr">
-        <is>
-          <t>Come either today or tomorrow.</t>
-        </is>
-      </c>
+      <c r="W69" s="13" t="inlineStr"/>
       <c r="X69" s="13" t="inlineStr">
         <is>
           <t>Ya toh aaj aao ya kal.</t>
@@ -15494,14 +15450,10 @@
       </c>
       <c r="V71" s="14" t="inlineStr">
         <is>
-          <t>English is spoken here.</t>
-        </is>
-      </c>
-      <c r="W71" s="14" t="inlineStr">
-        <is>
           <t>Rice is grown in Punjab.</t>
         </is>
       </c>
+      <c r="W71" s="13" t="inlineStr"/>
       <c r="X71" s="13" t="inlineStr">
         <is>
           <t>Yahan English boli jaati hai.</t>
@@ -15698,14 +15650,10 @@
       </c>
       <c r="V72" s="14" t="inlineStr">
         <is>
-          <t>This house was built in 1990.</t>
-        </is>
-      </c>
-      <c r="W72" s="14" t="inlineStr">
-        <is>
           <t>The Taj Mahal was built by Shah Jahan.</t>
         </is>
       </c>
+      <c r="W72" s="13" t="inlineStr"/>
       <c r="X72" s="13" t="inlineStr">
         <is>
           <t>Yeh ghar 1990 mein banaya gaya tha.</t>
@@ -16522,14 +16470,10 @@
       </c>
       <c r="V76" s="14" t="inlineStr">
         <is>
-          <t>He asked me to wait.</t>
-        </is>
-      </c>
-      <c r="W76" s="14" t="inlineStr">
-        <is>
           <t>She asked me to help.</t>
         </is>
       </c>
+      <c r="W76" s="13" t="inlineStr"/>
       <c r="X76" s="13" t="inlineStr">
         <is>
           <t>Usne mujhse wait karne ko kaha.</t>
@@ -16942,14 +16886,10 @@
       </c>
       <c r="V78" s="14" t="inlineStr">
         <is>
-          <t>I don't know what his name is.</t>
-        </is>
-      </c>
-      <c r="W78" s="14" t="inlineStr">
-        <is>
           <t>I don't know what time it is.</t>
         </is>
       </c>
+      <c r="W78" s="13" t="inlineStr"/>
       <c r="X78" s="13" t="inlineStr">
         <is>
           <t>Mujhe nahi pata ki uska naam kya hai.</t>
@@ -17150,14 +17090,10 @@
       </c>
       <c r="V79" s="14" t="inlineStr">
         <is>
-          <t>I'm sure you'll pass.</t>
-        </is>
-      </c>
-      <c r="W79" s="14" t="inlineStr">
-        <is>
           <t>I'm sure he's home.</t>
         </is>
       </c>
+      <c r="W79" s="13" t="inlineStr"/>
       <c r="X79" s="13" t="inlineStr">
         <is>
           <t>Mujhe yakeen hai ki tum pass ho jaoge.</t>
@@ -17366,14 +17302,10 @@
       </c>
       <c r="V80" s="14" t="inlineStr">
         <is>
-          <t>I don't think he'll come.</t>
-        </is>
-      </c>
-      <c r="W80" s="14" t="inlineStr">
-        <is>
           <t>I don't think it's true.</t>
         </is>
       </c>
+      <c r="W80" s="13" t="inlineStr"/>
       <c r="X80" s="13" t="inlineStr">
         <is>
           <t>Mujhe nahi lagta ki woh aayega.</t>
@@ -17574,14 +17506,10 @@
       </c>
       <c r="V81" s="14" t="inlineStr">
         <is>
-          <t>I hope you get the job.</t>
-        </is>
-      </c>
-      <c r="W81" s="14" t="inlineStr">
-        <is>
           <t>I hope it doesn't rain.</t>
         </is>
       </c>
+      <c r="W81" s="13" t="inlineStr"/>
       <c r="X81" s="13" t="inlineStr">
         <is>
           <t>Mujhe ummeed hai ki tumhe job mil jaaye.</t>
@@ -18006,14 +17934,10 @@
       </c>
       <c r="V83" s="14" t="inlineStr">
         <is>
-          <t>Dad let me go.</t>
-        </is>
-      </c>
-      <c r="W83" s="14" t="inlineStr">
-        <is>
           <t>She let me use her phone.</t>
         </is>
       </c>
+      <c r="W83" s="13" t="inlineStr"/>
       <c r="X83" s="13" t="inlineStr">
         <is>
           <t>Papa ne mujhe jaane diya.</t>
@@ -19466,14 +19390,10 @@
       </c>
       <c r="V90" s="14" t="inlineStr">
         <is>
-          <t>Should I call him?</t>
-        </is>
-      </c>
-      <c r="W90" s="14" t="inlineStr">
-        <is>
           <t>Should I take the job?</t>
         </is>
       </c>
+      <c r="W90" s="13" t="inlineStr"/>
       <c r="X90" s="13" t="inlineStr">
         <is>
           <t>Kya mujhe usse call karna chahiye?</t>
@@ -19882,14 +19802,10 @@
       </c>
       <c r="V92" s="14" t="inlineStr">
         <is>
-          <t>I had to walk.</t>
-        </is>
-      </c>
-      <c r="W92" s="14" t="inlineStr">
-        <is>
           <t>I had to wait an hour.</t>
         </is>
       </c>
+      <c r="W92" s="13" t="inlineStr"/>
       <c r="X92" s="13" t="inlineStr">
         <is>
           <t>Mujhe paidal jaana pada.</t>
@@ -20730,14 +20646,10 @@
       </c>
       <c r="V96" s="14" t="inlineStr">
         <is>
-          <t>You must visit Goa.</t>
-        </is>
-      </c>
-      <c r="W96" s="14" t="inlineStr">
-        <is>
           <t>You must wear a helmet.</t>
         </is>
       </c>
+      <c r="W96" s="13" t="inlineStr"/>
       <c r="X96" s="13" t="inlineStr">
         <is>
           <t>Tum zaroor Goa jaana.</t>
@@ -21570,14 +21482,10 @@
       </c>
       <c r="V100" s="14" t="inlineStr">
         <is>
-          <t>I've finished packing.</t>
-        </is>
-      </c>
-      <c r="W100" s="14" t="inlineStr">
-        <is>
           <t>I've finished eating.</t>
         </is>
       </c>
+      <c r="W100" s="13" t="inlineStr"/>
       <c r="X100" s="13" t="inlineStr">
         <is>
           <t>Maine packing khatam kar li.</t>
@@ -21781,11 +21689,7 @@
           <t>I forgot to call.</t>
         </is>
       </c>
-      <c r="W101" s="14" t="inlineStr">
-        <is>
-          <t>I forgot to lock the door.</t>
-        </is>
-      </c>
+      <c r="W101" s="13" t="inlineStr"/>
       <c r="X101" s="13" t="inlineStr">
         <is>
           <t>Main darwaza lock karna bhool gaya.</t>
@@ -21990,14 +21894,10 @@
       </c>
       <c r="V102" s="14" t="inlineStr">
         <is>
-          <t>I'm learning to drive.</t>
-        </is>
-      </c>
-      <c r="W102" s="14" t="inlineStr">
-        <is>
           <t>She's learning to swim.</t>
         </is>
       </c>
+      <c r="W102" s="13" t="inlineStr"/>
       <c r="X102" s="13" t="inlineStr">
         <is>
           <t>Main gaadi chalana seekh raha hoon.</t>
@@ -22202,14 +22102,10 @@
       </c>
       <c r="V103" s="14" t="inlineStr">
         <is>
-          <t>I started going to the gym.</t>
-        </is>
-      </c>
-      <c r="W103" s="14" t="inlineStr">
-        <is>
           <t>She started learning Hindi.</t>
         </is>
       </c>
+      <c r="W103" s="13" t="inlineStr"/>
       <c r="X103" s="13" t="inlineStr">
         <is>
           <t>Maine gym jaana shuru kiya.</t>
@@ -23253,11 +23149,7 @@
           <t>I'm scared to fly.</t>
         </is>
       </c>
-      <c r="W108" s="14" t="inlineStr">
-        <is>
-          <t>I'm scared to speak on stage.</t>
-        </is>
-      </c>
+      <c r="W108" s="13" t="inlineStr"/>
       <c r="X108" s="13" t="inlineStr">
         <is>
           <t>Main stage par bolne se darta hoon.</t>
@@ -23678,14 +23570,10 @@
       </c>
       <c r="V110" s="14" t="inlineStr">
         <is>
-          <t>I'm glad to hear that.</t>
-        </is>
-      </c>
-      <c r="W110" s="14" t="inlineStr">
-        <is>
           <t>I'm glad to help.</t>
         </is>
       </c>
+      <c r="W110" s="13" t="inlineStr"/>
       <c r="X110" s="13" t="inlineStr">
         <is>
           <t>Mujhe yeh sunkar khushi hui.</t>
@@ -24529,11 +24417,7 @@
           <t>How do you cook dal?</t>
         </is>
       </c>
-      <c r="W114" s="14" t="inlineStr">
-        <is>
-          <t>How do you practise English?</t>
-        </is>
-      </c>
+      <c r="W114" s="13" t="inlineStr"/>
       <c r="X114" s="13" t="inlineStr">
         <is>
           <t>Tum English kaise practise karte ho?</t>
@@ -24949,11 +24833,7 @@
           <t>Why are you crying?</t>
         </is>
       </c>
-      <c r="W116" s="14" t="inlineStr">
-        <is>
-          <t>Why are you laughing?</t>
-        </is>
-      </c>
+      <c r="W116" s="13" t="inlineStr"/>
       <c r="X116" s="13" t="inlineStr">
         <is>
           <t>Tum has kyon rahe ho?</t>
@@ -25370,14 +25250,10 @@
       </c>
       <c r="V118" s="14" t="inlineStr">
         <is>
-          <t>Why do you like cricket?</t>
-        </is>
-      </c>
-      <c r="W118" s="14" t="inlineStr">
-        <is>
           <t>Why do you like this song?</t>
         </is>
       </c>
+      <c r="W118" s="13" t="inlineStr"/>
       <c r="X118" s="13" t="inlineStr">
         <is>
           <t>Tumhe cricket kyon pasand hai?</t>
@@ -25578,14 +25454,10 @@
       </c>
       <c r="V119" s="14" t="inlineStr">
         <is>
-          <t>Do you think it will rain?</t>
-        </is>
-      </c>
-      <c r="W119" s="14" t="inlineStr">
-        <is>
           <t>Do you think he's right?</t>
         </is>
       </c>
+      <c r="W119" s="13" t="inlineStr"/>
       <c r="X119" s="13" t="inlineStr">
         <is>
           <t>Tumhe kya lagta hai, baarish hogi?</t>
@@ -25790,14 +25662,10 @@
       </c>
       <c r="V120" s="14" t="inlineStr">
         <is>
-          <t>Which is better, tea or coffee?</t>
-        </is>
-      </c>
-      <c r="W120" s="14" t="inlineStr">
-        <is>
           <t>Which is better, this or that?</t>
         </is>
       </c>
+      <c r="W120" s="13" t="inlineStr"/>
       <c r="X120" s="13" t="inlineStr">
         <is>
           <t>Kaunsa behtar hai, chai ya coffee?</t>
@@ -26002,14 +25870,10 @@
       </c>
       <c r="V121" s="14" t="inlineStr">
         <is>
-          <t>Which phone is the best?</t>
-        </is>
-      </c>
-      <c r="W121" s="14" t="inlineStr">
-        <is>
           <t>Which school is the best?</t>
         </is>
       </c>
+      <c r="W121" s="13" t="inlineStr"/>
       <c r="X121" s="13" t="inlineStr">
         <is>
           <t>Kaunsa phone sabse achha hai?</t>
@@ -26218,14 +26082,10 @@
       </c>
       <c r="V122" s="14" t="inlineStr">
         <is>
-          <t>I haven't eaten yet.</t>
-        </is>
-      </c>
-      <c r="W122" s="14" t="inlineStr">
-        <is>
           <t>I haven't finished yet.</t>
         </is>
       </c>
+      <c r="W122" s="13" t="inlineStr"/>
       <c r="X122" s="13" t="inlineStr">
         <is>
           <t>Maine abhi tak khana nahi khaya.</t>
@@ -26634,14 +26494,10 @@
       </c>
       <c r="V124" s="14" t="inlineStr">
         <is>
-          <t>Were you sleeping?</t>
-        </is>
-      </c>
-      <c r="W124" s="14" t="inlineStr">
-        <is>
           <t>Were you working at 6?</t>
         </is>
       </c>
+      <c r="W124" s="13" t="inlineStr"/>
       <c r="X124" s="13" t="inlineStr">
         <is>
           <t>Kya tum so rahe the?</t>
@@ -27474,14 +27330,10 @@
       </c>
       <c r="V128" s="14" t="inlineStr">
         <is>
-          <t>Whenever I meet him, he smiles.</t>
-        </is>
-      </c>
-      <c r="W128" s="14" t="inlineStr">
-        <is>
           <t>Whenever it rains, I stay in.</t>
         </is>
       </c>
+      <c r="W128" s="13" t="inlineStr"/>
       <c r="X128" s="13" t="inlineStr">
         <is>
           <t>Jab bhi main usse milta hoon, woh muskurata hai.</t>
@@ -28530,14 +28382,10 @@
       </c>
       <c r="V133" s="14" t="inlineStr">
         <is>
-          <t>It's time to sleep.</t>
-        </is>
-      </c>
-      <c r="W133" s="14" t="inlineStr">
-        <is>
           <t>It's time to go.</t>
         </is>
       </c>
+      <c r="W133" s="13" t="inlineStr"/>
       <c r="X133" s="13" t="inlineStr">
         <is>
           <t>Sone ka time ho gaya hai.</t>
@@ -29166,14 +29014,10 @@
       </c>
       <c r="V136" s="14" t="inlineStr">
         <is>
-          <t>There's no need to worry.</t>
-        </is>
-      </c>
-      <c r="W136" s="14" t="inlineStr">
-        <is>
           <t>There's no need to shout.</t>
         </is>
       </c>
+      <c r="W136" s="13" t="inlineStr"/>
       <c r="X136" s="13" t="inlineStr">
         <is>
           <t>Chinta karne ki koi zaroorat nahi.</t>
@@ -29378,14 +29222,10 @@
       </c>
       <c r="V137" s="14" t="inlineStr">
         <is>
-          <t>It's good that you came.</t>
-        </is>
-      </c>
-      <c r="W137" s="14" t="inlineStr">
-        <is>
           <t>It's good that it stopped raining.</t>
         </is>
       </c>
+      <c r="W137" s="13" t="inlineStr"/>
       <c r="X137" s="13" t="inlineStr">
         <is>
           <t>Yeh achha hai ki tum aa gaye.</t>
@@ -30226,14 +30066,10 @@
       </c>
       <c r="V141" s="14" t="inlineStr">
         <is>
-          <t>I like both tea and coffee.</t>
-        </is>
-      </c>
-      <c r="W141" s="14" t="inlineStr">
-        <is>
           <t>She likes both dogs and cats.</t>
         </is>
       </c>
+      <c r="W141" s="13" t="inlineStr"/>
       <c r="X141" s="13" t="inlineStr">
         <is>
           <t>Mujhe chai aur coffee dono pasand hain.</t>
@@ -30441,11 +30277,7 @@
           <t>Come as soon as possible.</t>
         </is>
       </c>
-      <c r="W142" s="14" t="inlineStr">
-        <is>
-          <t>Practise as much as possible.</t>
-        </is>
-      </c>
+      <c r="W142" s="13" t="inlineStr"/>
       <c r="X142" s="13" t="inlineStr">
         <is>
           <t>Jitna ho sake utna practice karo.</t>
@@ -31103,13 +30935,21 @@
           <t>Main bees minute se intezaar kar raha hoon.</t>
         </is>
       </c>
-      <c r="Y145" s="13" t="inlineStr">
-        <is>
-          <t>Present perfect continuous</t>
-        </is>
-      </c>
-      <c r="Z145" s="13" t="inlineStr"/>
-      <c r="AA145" s="13" t="inlineStr"/>
+      <c r="Y145" s="14" t="inlineStr">
+        <is>
+          <t>I am waiting since one hour.</t>
+        </is>
+      </c>
+      <c r="Z145" s="14" t="inlineStr">
+        <is>
+          <t>I have been waiting for an hour.</t>
+        </is>
+      </c>
+      <c r="AA145" s="14" t="inlineStr">
+        <is>
+          <t>Use present perfect continuous, not present.</t>
+        </is>
+      </c>
       <c r="AB145" s="14" t="inlineStr">
         <is>
           <t>have/has been + -ing + for/since.</t>
@@ -32154,14 +31994,10 @@
       </c>
       <c r="V150" s="14" t="inlineStr">
         <is>
-          <t>I keep forgetting names.</t>
-        </is>
-      </c>
-      <c r="W150" s="14" t="inlineStr">
-        <is>
           <t>I keep losing my keys.</t>
         </is>
       </c>
+      <c r="W150" s="13" t="inlineStr"/>
       <c r="X150" s="13" t="inlineStr">
         <is>
           <t>Main naam bhoolta rehta hoon.</t>
@@ -32570,14 +32406,10 @@
       </c>
       <c r="V152" s="14" t="inlineStr">
         <is>
-          <t>The train had already left before I arrived.</t>
-        </is>
-      </c>
-      <c r="W152" s="14" t="inlineStr">
-        <is>
           <t>The film had started before we came.</t>
         </is>
       </c>
+      <c r="W152" s="13" t="inlineStr"/>
       <c r="X152" s="13" t="inlineStr">
         <is>
           <t>Mere pahunchne se pehle hi train ja chuki thi.</t>
@@ -32789,11 +32621,7 @@
           <t>I'm thinking of buying a car.</t>
         </is>
       </c>
-      <c r="W153" s="14" t="inlineStr">
-        <is>
-          <t>I'm thinking of doing an MBA.</t>
-        </is>
-      </c>
+      <c r="W153" s="13" t="inlineStr"/>
       <c r="X153" s="13" t="inlineStr">
         <is>
           <t>Main MBA karne ka soch raha hoon.</t>
@@ -34041,11 +33869,7 @@
           <t>How long have you been waiting?</t>
         </is>
       </c>
-      <c r="W159" s="14" t="inlineStr">
-        <is>
-          <t>How long have you been learning English?</t>
-        </is>
-      </c>
+      <c r="W159" s="13" t="inlineStr"/>
       <c r="X159" s="13" t="inlineStr">
         <is>
           <t>Tum kab se English seekh rahe ho?</t>
@@ -34870,14 +34694,10 @@
       </c>
       <c r="V163" s="14" t="inlineStr">
         <is>
-          <t>I like neither tea nor coffee.</t>
-        </is>
-      </c>
-      <c r="W163" s="14" t="inlineStr">
-        <is>
           <t>He's neither rich nor poor.</t>
         </is>
       </c>
+      <c r="W163" s="13" t="inlineStr"/>
       <c r="X163" s="13" t="inlineStr">
         <is>
           <t>Mujhe na chai pasand hai na coffee.</t>
@@ -35074,14 +34894,10 @@
       </c>
       <c r="V164" s="14" t="inlineStr">
         <is>
-          <t>The result will be announced tomorrow.</t>
-        </is>
-      </c>
-      <c r="W164" s="14" t="inlineStr">
-        <is>
           <t>The work will be done by Friday.</t>
         </is>
       </c>
+      <c r="W164" s="13" t="inlineStr"/>
       <c r="X164" s="13" t="inlineStr">
         <is>
           <t>Result kal ghoshit kiya jaayega.</t>
@@ -35282,14 +35098,10 @@
       </c>
       <c r="V165" s="14" t="inlineStr">
         <is>
-          <t>Your order has been sent.</t>
-        </is>
-      </c>
-      <c r="W165" s="14" t="inlineStr">
-        <is>
           <t>The room has been cleaned.</t>
         </is>
       </c>
+      <c r="W165" s="13" t="inlineStr"/>
       <c r="X165" s="13" t="inlineStr">
         <is>
           <t>Aapka order bhej diya gaya hai.</t>
@@ -35898,14 +35710,10 @@
       </c>
       <c r="V168" s="14" t="inlineStr">
         <is>
-          <t>This rule should be changed.</t>
-        </is>
-      </c>
-      <c r="W168" s="14" t="inlineStr">
-        <is>
           <t>Waste should be recycled.</t>
         </is>
       </c>
+      <c r="W168" s="13" t="inlineStr"/>
       <c r="X168" s="13" t="inlineStr">
         <is>
           <t>Is niyam ko badla jaana chahiye.</t>
@@ -36310,14 +36118,10 @@
       </c>
       <c r="V170" s="14" t="inlineStr">
         <is>
-          <t>I was given a certificate.</t>
-        </is>
-      </c>
-      <c r="W170" s="14" t="inlineStr">
-        <is>
           <t>I was given a chance.</t>
         </is>
       </c>
+      <c r="W170" s="13" t="inlineStr"/>
       <c r="X170" s="13" t="inlineStr">
         <is>
           <t>Mujhe ek certificate diya gaya.</t>
@@ -36730,14 +36534,10 @@
       </c>
       <c r="V172" s="14" t="inlineStr">
         <is>
-          <t>He told me not to come late.</t>
-        </is>
-      </c>
-      <c r="W172" s="14" t="inlineStr">
-        <is>
           <t>Mum told me not to worry.</t>
         </is>
       </c>
+      <c r="W172" s="13" t="inlineStr"/>
       <c r="X172" s="13" t="inlineStr">
         <is>
           <t>Usne mujhse late na aane ko kaha.</t>
@@ -36938,14 +36738,10 @@
       </c>
       <c r="V173" s="14" t="inlineStr">
         <is>
-          <t>He asked if I was free.</t>
-        </is>
-      </c>
-      <c r="W173" s="14" t="inlineStr">
-        <is>
           <t>She asked if we were coming.</t>
         </is>
       </c>
+      <c r="W173" s="13" t="inlineStr"/>
       <c r="X173" s="13" t="inlineStr">
         <is>
           <t>Usne poocha ki kya main free hoon.</t>
@@ -37146,14 +36942,10 @@
       </c>
       <c r="V174" s="14" t="inlineStr">
         <is>
-          <t>He asked where the station was.</t>
-        </is>
-      </c>
-      <c r="W174" s="14" t="inlineStr">
-        <is>
           <t>She asked where I lived.</t>
         </is>
       </c>
+      <c r="W174" s="13" t="inlineStr"/>
       <c r="X174" s="13" t="inlineStr">
         <is>
           <t>Usne poocha ki station kahan hai.</t>
@@ -37982,14 +37774,10 @@
       </c>
       <c r="V178" s="14" t="inlineStr">
         <is>
-          <t>Could you tell me when the bank opens?</t>
-        </is>
-      </c>
-      <c r="W178" s="14" t="inlineStr">
-        <is>
           <t>Could you tell me where the lift is?</t>
         </is>
       </c>
+      <c r="W178" s="13" t="inlineStr"/>
       <c r="X178" s="13" t="inlineStr">
         <is>
           <t>Kya aap bata sakte hain ki bank kab khulta hai?</t>
@@ -38186,14 +37974,10 @@
       </c>
       <c r="V179" s="14" t="inlineStr">
         <is>
-          <t>What I need is some rest.</t>
-        </is>
-      </c>
-      <c r="W179" s="14" t="inlineStr">
-        <is>
           <t>What I need is a good job.</t>
         </is>
       </c>
+      <c r="W179" s="13" t="inlineStr"/>
       <c r="X179" s="13" t="inlineStr">
         <is>
           <t>Mujhe jo chahiye woh hai thoda aaraam.</t>
@@ -38822,14 +38606,10 @@
       </c>
       <c r="V182" s="14" t="inlineStr">
         <is>
-          <t>The doctor advised me to rest.</t>
-        </is>
-      </c>
-      <c r="W182" s="14" t="inlineStr">
-        <is>
           <t>She advised me to wait.</t>
         </is>
       </c>
+      <c r="W182" s="13" t="inlineStr"/>
       <c r="X182" s="13" t="inlineStr">
         <is>
           <t>Doctor ne mujhe aaraam karne ki salah di.</t>
@@ -39234,14 +39014,10 @@
       </c>
       <c r="V184" s="14" t="inlineStr">
         <is>
-          <t>I got my phone repaired.</t>
-        </is>
-      </c>
-      <c r="W184" s="14" t="inlineStr">
-        <is>
           <t>I got my hair cut.</t>
         </is>
       </c>
+      <c r="W184" s="13" t="inlineStr"/>
       <c r="X184" s="13" t="inlineStr">
         <is>
           <t>Maine apna phone theek karwaya.</t>
@@ -39438,14 +39214,10 @@
       </c>
       <c r="V185" s="14" t="inlineStr">
         <is>
-          <t>I have my hair cut every month.</t>
-        </is>
-      </c>
-      <c r="W185" s="14" t="inlineStr">
-        <is>
           <t>I have my car washed weekly.</t>
         </is>
       </c>
+      <c r="W185" s="13" t="inlineStr"/>
       <c r="X185" s="13" t="inlineStr">
         <is>
           <t>Main har mahine baal katwata hoon.</t>
@@ -39642,14 +39414,10 @@
       </c>
       <c r="V186" s="14" t="inlineStr">
         <is>
-          <t>My boss allowed me to work from home.</t>
-        </is>
-      </c>
-      <c r="W186" s="14" t="inlineStr">
-        <is>
           <t>Dad allowed me to go.</t>
         </is>
       </c>
+      <c r="W186" s="13" t="inlineStr"/>
       <c r="X186" s="13" t="inlineStr">
         <is>
           <t>Boss ne mujhe ghar se kaam karne ki ijazat di.</t>
@@ -40062,14 +39830,10 @@
       </c>
       <c r="V188" s="14" t="inlineStr">
         <is>
-          <t>He must be tired.</t>
-        </is>
-      </c>
-      <c r="W188" s="14" t="inlineStr">
-        <is>
           <t>She must be at home.</t>
         </is>
       </c>
+      <c r="W188" s="13" t="inlineStr"/>
       <c r="X188" s="13" t="inlineStr">
         <is>
           <t>Woh zaroor thaka hoga.</t>
@@ -40478,14 +40242,10 @@
       </c>
       <c r="V190" s="14" t="inlineStr">
         <is>
-          <t>He can't be at the office now.</t>
-        </is>
-      </c>
-      <c r="W190" s="14" t="inlineStr">
-        <is>
           <t>That can't be true.</t>
         </is>
       </c>
+      <c r="W190" s="13" t="inlineStr"/>
       <c r="X190" s="13" t="inlineStr">
         <is>
           <t>Woh abhi office mein nahi ho sakta.</t>
@@ -40686,14 +40446,10 @@
       </c>
       <c r="V191" s="14" t="inlineStr">
         <is>
-          <t>He must have missed the train.</t>
-        </is>
-      </c>
-      <c r="W191" s="14" t="inlineStr">
-        <is>
           <t>She must have forgotten.</t>
         </is>
       </c>
+      <c r="W191" s="13" t="inlineStr"/>
       <c r="X191" s="13" t="inlineStr">
         <is>
           <t>Usne zaroor train miss kar di hogi.</t>
@@ -40898,14 +40654,10 @@
       </c>
       <c r="V192" s="14" t="inlineStr">
         <is>
-          <t>He might have forgotten.</t>
-        </is>
-      </c>
-      <c r="W192" s="14" t="inlineStr">
-        <is>
           <t>She might have left.</t>
         </is>
       </c>
+      <c r="W192" s="13" t="inlineStr"/>
       <c r="X192" s="13" t="inlineStr">
         <is>
           <t>Shayad woh bhool gaya ho.</t>
@@ -41110,14 +40862,10 @@
       </c>
       <c r="V193" s="14" t="inlineStr">
         <is>
-          <t>He can't have done this alone.</t>
-        </is>
-      </c>
-      <c r="W193" s="14" t="inlineStr">
-        <is>
           <t>She can't have forgotten.</t>
         </is>
       </c>
+      <c r="W193" s="13" t="inlineStr"/>
       <c r="X193" s="13" t="inlineStr">
         <is>
           <t>Usne yeh akele nahi kiya hoga.</t>
@@ -41318,14 +41066,10 @@
       </c>
       <c r="V194" s="14" t="inlineStr">
         <is>
-          <t>I could have won.</t>
-        </is>
-      </c>
-      <c r="W194" s="14" t="inlineStr">
-        <is>
           <t>You could have told me.</t>
         </is>
       </c>
+      <c r="W194" s="13" t="inlineStr"/>
       <c r="X194" s="13" t="inlineStr">
         <is>
           <t>Main jeet sakta tha.</t>
@@ -41734,14 +41478,10 @@
       </c>
       <c r="V196" s="14" t="inlineStr">
         <is>
-          <t>I shouldn't have eaten so much.</t>
-        </is>
-      </c>
-      <c r="W196" s="14" t="inlineStr">
-        <is>
           <t>I shouldn't have shouted.</t>
         </is>
       </c>
+      <c r="W196" s="13" t="inlineStr"/>
       <c r="X196" s="13" t="inlineStr">
         <is>
           <t>Mujhe itna nahi khana chahiye tha.</t>
@@ -41950,14 +41690,10 @@
       </c>
       <c r="V197" s="14" t="inlineStr">
         <is>
-          <t>You'd better leave now.</t>
-        </is>
-      </c>
-      <c r="W197" s="14" t="inlineStr">
-        <is>
           <t>You'd better study.</t>
         </is>
       </c>
+      <c r="W197" s="13" t="inlineStr"/>
       <c r="X197" s="13" t="inlineStr">
         <is>
           <t>Behtar hoga ki tum abhi nikal jao.</t>
@@ -42366,14 +42102,10 @@
       </c>
       <c r="V199" s="14" t="inlineStr">
         <is>
-          <t>You didn't need to bring a gift.</t>
-        </is>
-      </c>
-      <c r="W199" s="14" t="inlineStr">
-        <is>
           <t>You didn't need to wait.</t>
         </is>
       </c>
+      <c r="W199" s="13" t="inlineStr"/>
       <c r="X199" s="13" t="inlineStr">
         <is>
           <t>Tumhe gift laane ki zaroorat nahi thi.</t>
@@ -42578,14 +42310,10 @@
       </c>
       <c r="V200" s="14" t="inlineStr">
         <is>
-          <t>He might not come.</t>
-        </is>
-      </c>
-      <c r="W200" s="14" t="inlineStr">
-        <is>
           <t>It might not rain.</t>
         </is>
       </c>
+      <c r="W200" s="13" t="inlineStr"/>
       <c r="X200" s="13" t="inlineStr">
         <is>
           <t>Ho sakta hai ki woh na aaye.</t>
@@ -42790,14 +42518,10 @@
       </c>
       <c r="V201" s="14" t="inlineStr">
         <is>
-          <t>The train should arrive by five.</t>
-        </is>
-      </c>
-      <c r="W201" s="14" t="inlineStr">
-        <is>
           <t>The parcel should come by Friday.</t>
         </is>
       </c>
+      <c r="W201" s="13" t="inlineStr"/>
       <c r="X201" s="13" t="inlineStr">
         <is>
           <t>Train ko paanch baje tak aa jaana chahiye.</t>
@@ -42994,14 +42718,10 @@
       </c>
       <c r="V202" s="14" t="inlineStr">
         <is>
-          <t>I have no choice but to apologise.</t>
-        </is>
-      </c>
-      <c r="W202" s="14" t="inlineStr">
-        <is>
           <t>We had no choice but to wait.</t>
         </is>
       </c>
+      <c r="W202" s="13" t="inlineStr"/>
       <c r="X202" s="13" t="inlineStr">
         <is>
           <t>Mujhe maafi maangni hi padegi.</t>
@@ -43622,14 +43342,10 @@
       </c>
       <c r="V205" s="14" t="inlineStr">
         <is>
-          <t>I promised to call him.</t>
-        </is>
-      </c>
-      <c r="W205" s="14" t="inlineStr">
-        <is>
           <t>She promised to help.</t>
         </is>
       </c>
+      <c r="W205" s="13" t="inlineStr"/>
       <c r="X205" s="13" t="inlineStr">
         <is>
           <t>Maine usse call karne ka waada kiya.</t>
@@ -43834,14 +43550,10 @@
       </c>
       <c r="V206" s="14" t="inlineStr">
         <is>
-          <t>He refused to take the money.</t>
-        </is>
-      </c>
-      <c r="W206" s="14" t="inlineStr">
-        <is>
           <t>She refused to answer.</t>
         </is>
       </c>
+      <c r="W206" s="13" t="inlineStr"/>
       <c r="X206" s="13" t="inlineStr">
         <is>
           <t>Usne paise lene se mana kar diya.</t>
@@ -44254,14 +43966,10 @@
       </c>
       <c r="V208" s="14" t="inlineStr">
         <is>
-          <t>I find it hard to get up early.</t>
-        </is>
-      </c>
-      <c r="W208" s="14" t="inlineStr">
-        <is>
           <t>I find it hard to focus.</t>
         </is>
       </c>
+      <c r="W208" s="13" t="inlineStr"/>
       <c r="X208" s="13" t="inlineStr">
         <is>
           <t>Mujhe subah jaldi uthne mein mushkil hoti hai.</t>
@@ -44462,14 +44170,10 @@
       </c>
       <c r="V209" s="14" t="inlineStr">
         <is>
-          <t>I got a chance to go to London.</t>
-        </is>
-      </c>
-      <c r="W209" s="14" t="inlineStr">
-        <is>
           <t>I got a chance to meet her.</t>
         </is>
       </c>
+      <c r="W209" s="13" t="inlineStr"/>
       <c r="X209" s="13" t="inlineStr">
         <is>
           <t>Mujhe London jaane ka mauka mila.</t>
@@ -44678,14 +44382,10 @@
       </c>
       <c r="V210" s="14" t="inlineStr">
         <is>
-          <t>I don't mind waiting.</t>
-        </is>
-      </c>
-      <c r="W210" s="14" t="inlineStr">
-        <is>
           <t>I don't mind helping.</t>
         </is>
       </c>
+      <c r="W210" s="13" t="inlineStr"/>
       <c r="X210" s="13" t="inlineStr">
         <is>
           <t>Mujhe wait karne mein koi dikkat nahi.</t>
@@ -44886,14 +44586,10 @@
       </c>
       <c r="V211" s="14" t="inlineStr">
         <is>
-          <t>I tried restarting the phone.</t>
-        </is>
-      </c>
-      <c r="W211" s="14" t="inlineStr">
-        <is>
           <t>Try adding more salt.</t>
         </is>
       </c>
+      <c r="W211" s="13" t="inlineStr"/>
       <c r="X211" s="13" t="inlineStr">
         <is>
           <t>Maine phone restart karke dekha.</t>
@@ -45090,14 +44786,10 @@
       </c>
       <c r="V212" s="14" t="inlineStr">
         <is>
-          <t>I regret lying to him.</t>
-        </is>
-      </c>
-      <c r="W212" s="14" t="inlineStr">
-        <is>
           <t>I regret not studying.</t>
         </is>
       </c>
+      <c r="W212" s="13" t="inlineStr"/>
       <c r="X212" s="13" t="inlineStr">
         <is>
           <t>Mujhe usse jhooth bolne ka pachhtava hai.</t>
@@ -45302,14 +44994,10 @@
       </c>
       <c r="V213" s="14" t="inlineStr">
         <is>
-          <t>I'm determined to learn English.</t>
-        </is>
-      </c>
-      <c r="W213" s="14" t="inlineStr">
-        <is>
           <t>She's determined to win.</t>
         </is>
       </c>
+      <c r="W213" s="13" t="inlineStr"/>
       <c r="X213" s="13" t="inlineStr">
         <is>
           <t>Maine English seekhne ki thaan li hai.</t>
@@ -45730,14 +45418,10 @@
       </c>
       <c r="V215" s="14" t="inlineStr">
         <is>
-          <t>I'll give up smoking.</t>
-        </is>
-      </c>
-      <c r="W215" s="14" t="inlineStr">
-        <is>
           <t>I'll give up eating sugar.</t>
         </is>
       </c>
+      <c r="W215" s="13" t="inlineStr"/>
       <c r="X215" s="13" t="inlineStr">
         <is>
           <t>Main smoking chhod dunga.</t>
@@ -45938,14 +45622,10 @@
       </c>
       <c r="V216" s="14" t="inlineStr">
         <is>
-          <t>I suggest leaving early.</t>
-        </is>
-      </c>
-      <c r="W216" s="14" t="inlineStr">
-        <is>
           <t>I suggest trying this.</t>
         </is>
       </c>
+      <c r="W216" s="13" t="inlineStr"/>
       <c r="X216" s="13" t="inlineStr">
         <is>
           <t>Main suggest karta hoon ki hum jaldi niklein.</t>
@@ -46358,14 +46038,10 @@
       </c>
       <c r="V218" s="14" t="inlineStr">
         <is>
-          <t>I spent three hours learning this.</t>
-        </is>
-      </c>
-      <c r="W218" s="14" t="inlineStr">
-        <is>
           <t>I spent the day cooking.</t>
         </is>
       </c>
+      <c r="W218" s="13" t="inlineStr"/>
       <c r="X218" s="13" t="inlineStr">
         <is>
           <t>Maine yeh seekhne mein teen ghante bitaye.</t>
@@ -46566,14 +46242,10 @@
       </c>
       <c r="V219" s="14" t="inlineStr">
         <is>
-          <t>I had trouble finding the house.</t>
-        </is>
-      </c>
-      <c r="W219" s="14" t="inlineStr">
-        <is>
           <t>I had trouble sleeping.</t>
         </is>
       </c>
+      <c r="W219" s="13" t="inlineStr"/>
       <c r="X219" s="13" t="inlineStr">
         <is>
           <t>Mujhe ghar dhoondhne mein dikkat hui.</t>
@@ -46774,14 +46446,10 @@
       </c>
       <c r="V220" s="14" t="inlineStr">
         <is>
-          <t>I couldn't help laughing.</t>
-        </is>
-      </c>
-      <c r="W220" s="14" t="inlineStr">
-        <is>
           <t>I couldn't help crying.</t>
         </is>
       </c>
+      <c r="W220" s="13" t="inlineStr"/>
       <c r="X220" s="13" t="inlineStr">
         <is>
           <t>Main hasne se khud ko rok nahi paaya.</t>
@@ -46982,14 +46650,10 @@
       </c>
       <c r="V221" s="14" t="inlineStr">
         <is>
-          <t>Who made this?</t>
-        </is>
-      </c>
-      <c r="W221" s="14" t="inlineStr">
-        <is>
           <t>Who broke the glass?</t>
         </is>
       </c>
+      <c r="W221" s="13" t="inlineStr"/>
       <c r="X221" s="13" t="inlineStr">
         <is>
           <t>Yeh kisne banaya?</t>
@@ -47186,14 +46850,10 @@
       </c>
       <c r="V222" s="14" t="inlineStr">
         <is>
-          <t>What's the best way to learn English?</t>
-        </is>
-      </c>
-      <c r="W222" s="14" t="inlineStr">
-        <is>
           <t>What's the best way to get there?</t>
         </is>
       </c>
+      <c r="W222" s="13" t="inlineStr"/>
       <c r="X222" s="13" t="inlineStr">
         <is>
           <t>English seekhne ka sabse achha tareeka kya hai?</t>
@@ -47402,14 +47062,10 @@
       </c>
       <c r="V223" s="14" t="inlineStr">
         <is>
-          <t>What made you choose teaching?</t>
-        </is>
-      </c>
-      <c r="W223" s="14" t="inlineStr">
-        <is>
           <t>What made you choose this city?</t>
         </is>
       </c>
+      <c r="W223" s="13" t="inlineStr"/>
       <c r="X223" s="13" t="inlineStr">
         <is>
           <t>Tumne teaching kyon chuni?</t>
@@ -47606,14 +47262,10 @@
       </c>
       <c r="V224" s="14" t="inlineStr">
         <is>
-          <t>I haven't talked to him for two days.</t>
-        </is>
-      </c>
-      <c r="W224" s="14" t="inlineStr">
-        <is>
           <t>I haven't eaten for hours.</t>
         </is>
       </c>
+      <c r="W224" s="13" t="inlineStr"/>
       <c r="X224" s="13" t="inlineStr">
         <is>
           <t>Maine do din se usse baat nahi ki.</t>
@@ -47814,14 +47466,10 @@
       </c>
       <c r="V225" s="14" t="inlineStr">
         <is>
-          <t>It's been a year since I met him.</t>
-        </is>
-      </c>
-      <c r="W225" s="14" t="inlineStr">
-        <is>
           <t>It's been ages since I cooked.</t>
         </is>
       </c>
+      <c r="W225" s="13" t="inlineStr"/>
       <c r="X225" s="13" t="inlineStr">
         <is>
           <t>Usse mile hue ek saal ho gaya.</t>
@@ -48022,14 +47670,10 @@
       </c>
       <c r="V226" s="14" t="inlineStr">
         <is>
-          <t>I was going to call, but I forgot.</t>
-        </is>
-      </c>
-      <c r="W226" s="14" t="inlineStr">
-        <is>
           <t>I was going to cook, but I was tired.</t>
         </is>
       </c>
+      <c r="W226" s="13" t="inlineStr"/>
       <c r="X226" s="13" t="inlineStr">
         <is>
           <t>Main call karne wala tha, lekin bhool gaya.</t>
@@ -48234,14 +47878,10 @@
       </c>
       <c r="V227" s="14" t="inlineStr">
         <is>
-          <t>I had never flown before.</t>
-        </is>
-      </c>
-      <c r="W227" s="14" t="inlineStr">
-        <is>
           <t>She had never seen snow before.</t>
         </is>
       </c>
+      <c r="W227" s="13" t="inlineStr"/>
       <c r="X227" s="13" t="inlineStr">
         <is>
           <t>Maine pehle kabhi hawai jahaz mein safar nahi kiya tha.</t>
@@ -48650,14 +48290,10 @@
       </c>
       <c r="V229" s="14" t="inlineStr">
         <is>
-          <t>He's always complaining.</t>
-        </is>
-      </c>
-      <c r="W229" s="14" t="inlineStr">
-        <is>
           <t>She's always losing her keys.</t>
         </is>
       </c>
+      <c r="W229" s="13" t="inlineStr"/>
       <c r="X229" s="13" t="inlineStr">
         <is>
           <t>Woh hamesha shikayat karta rehta hai.</t>
@@ -48858,14 +48494,10 @@
       </c>
       <c r="V230" s="14" t="inlineStr">
         <is>
-          <t>I didn't use to drink tea.</t>
-        </is>
-      </c>
-      <c r="W230" s="14" t="inlineStr">
-        <is>
           <t>She didn't use to like maths.</t>
         </is>
       </c>
+      <c r="W230" s="13" t="inlineStr"/>
       <c r="X230" s="13" t="inlineStr">
         <is>
           <t>Main pehle chai nahi peeta tha.</t>
@@ -49062,14 +48694,10 @@
       </c>
       <c r="V231" s="14" t="inlineStr">
         <is>
-          <t>I had been waiting for an hour when he arrived.</t>
-        </is>
-      </c>
-      <c r="W231" s="14" t="inlineStr">
-        <is>
           <t>She had been working there for years when she left.</t>
         </is>
       </c>
+      <c r="W231" s="13" t="inlineStr"/>
       <c r="X231" s="13" t="inlineStr">
         <is>
           <t>Main ek ghante se wait kar raha tha, tab woh aaya.</t>
@@ -49474,14 +49102,10 @@
       </c>
       <c r="V233" s="14" t="inlineStr">
         <is>
-          <t>If I had studied, I would have passed.</t>
-        </is>
-      </c>
-      <c r="W233" s="14" t="inlineStr">
-        <is>
           <t>If you had called, I would have come.</t>
         </is>
       </c>
+      <c r="W233" s="13" t="inlineStr"/>
       <c r="X233" s="13" t="inlineStr">
         <is>
           <t>Agar maine padhai ki hoti, toh main pass ho jaata.</t>
@@ -49678,14 +49302,10 @@
       </c>
       <c r="V234" s="14" t="inlineStr">
         <is>
-          <t>As long as you work hard, you'll succeed.</t>
-        </is>
-      </c>
-      <c r="W234" s="14" t="inlineStr">
-        <is>
           <t>You can go, as long as you're back by 9.</t>
         </is>
       </c>
+      <c r="W234" s="13" t="inlineStr"/>
       <c r="X234" s="13" t="inlineStr">
         <is>
           <t>Jab tak tum mehnat karoge, tum safal hoge.</t>
@@ -50106,14 +49726,10 @@
       </c>
       <c r="V236" s="14" t="inlineStr">
         <is>
-          <t>Take an umbrella in case it rains.</t>
-        </is>
-      </c>
-      <c r="W236" s="14" t="inlineStr">
-        <is>
           <t>Save the file in case it crashes.</t>
         </is>
       </c>
+      <c r="W236" s="13" t="inlineStr"/>
       <c r="X236" s="13" t="inlineStr">
         <is>
           <t>Chhata le lo, kahin baarish na ho jaaye.</t>
@@ -50310,14 +49926,10 @@
       </c>
       <c r="V237" s="14" t="inlineStr">
         <is>
-          <t>Even if it rains, I'll come.</t>
-        </is>
-      </c>
-      <c r="W237" s="14" t="inlineStr">
-        <is>
           <t>Even if you shout, I won't go.</t>
         </is>
       </c>
+      <c r="W237" s="13" t="inlineStr"/>
       <c r="X237" s="13" t="inlineStr">
         <is>
           <t>Chahe baarish ho, main phir bhi aaunga.</t>
@@ -50522,14 +50134,10 @@
       </c>
       <c r="V238" s="14" t="inlineStr">
         <is>
-          <t>I wish I could speak French.</t>
-        </is>
-      </c>
-      <c r="W238" s="14" t="inlineStr">
-        <is>
           <t>I wish I could come.</t>
         </is>
       </c>
+      <c r="W238" s="13" t="inlineStr"/>
       <c r="X238" s="13" t="inlineStr">
         <is>
           <t>Kaash main French bol pata.</t>
@@ -50726,14 +50334,10 @@
       </c>
       <c r="V239" s="14" t="inlineStr">
         <is>
-          <t>I wish I had started earlier.</t>
-        </is>
-      </c>
-      <c r="W239" s="14" t="inlineStr">
-        <is>
           <t>I wish I had listened.</t>
         </is>
       </c>
+      <c r="W239" s="13" t="inlineStr"/>
       <c r="X239" s="13" t="inlineStr">
         <is>
           <t>Kaash maine pehle shuru kiya hota.</t>
@@ -51150,14 +50754,10 @@
       </c>
       <c r="V241" s="14" t="inlineStr">
         <is>
-          <t>Suppose you won the lottery, what would you do?</t>
-        </is>
-      </c>
-      <c r="W241" s="14" t="inlineStr">
-        <is>
           <t>Suppose it rained, what would we do?</t>
         </is>
       </c>
+      <c r="W241" s="13" t="inlineStr"/>
       <c r="X241" s="13" t="inlineStr">
         <is>
           <t>Maan lo ki tumhari lottery lag jaaye, toh kya karoge?</t>
@@ -51578,14 +51178,10 @@
       </c>
       <c r="V243" s="14" t="inlineStr">
         <is>
-          <t>This film is worth watching.</t>
-        </is>
-      </c>
-      <c r="W243" s="14" t="inlineStr">
-        <is>
           <t>It's worth trying.</t>
         </is>
       </c>
+      <c r="W243" s="13" t="inlineStr"/>
       <c r="X243" s="13" t="inlineStr">
         <is>
           <t>Yeh film dekhne layak hai.</t>
@@ -51994,14 +51590,10 @@
       </c>
       <c r="V245" s="14" t="inlineStr">
         <is>
-          <t>It doesn't matter where you're from.</t>
-        </is>
-      </c>
-      <c r="W245" s="14" t="inlineStr">
-        <is>
           <t>It doesn't matter if you're late.</t>
         </is>
       </c>
+      <c r="W245" s="13" t="inlineStr"/>
       <c r="X245" s="13" t="inlineStr">
         <is>
           <t>Koi fark nahi padta ki tum kahan se ho.</t>
@@ -52418,14 +52010,10 @@
       </c>
       <c r="V247" s="14" t="inlineStr">
         <is>
-          <t>It was such a good film that I watched it twice.</t>
-        </is>
-      </c>
-      <c r="W247" s="14" t="inlineStr">
-        <is>
           <t>She's such a kind person that everyone likes her.</t>
         </is>
       </c>
+      <c r="W247" s="13" t="inlineStr"/>
       <c r="X247" s="13" t="inlineStr">
         <is>
           <t>Woh itni achhi film thi ki maine do baar dekhi.</t>

</xml_diff>

<commit_message>
Third example for 632 cards; word audit fixes
- 632 chunk and grammar cards that lost a repeated example get a new third
  one (tools/rich/extra_ex_*.txt), so all 1,430 show three.
- Word audit: 36 words repeated an example sentence, and bring/last listed
  an opposite as a synonym. Fixed in word_fixes.py, applied on export.
- Review workbooks rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XivsNLnRJbP4wB6VLVY5B5
</commit_message>
<xml_diff>
--- a/content/chunk-library/Grammar_Library_Review.xlsx
+++ b/content/chunk-library/Grammar_Library_Review.xlsx
@@ -3841,7 +3841,11 @@
           <t>Will you come tomorrow?</t>
         </is>
       </c>
-      <c r="W16" s="13" t="inlineStr"/>
+      <c r="W16" s="14" t="inlineStr">
+        <is>
+          <t>Will you come to my birthday party?</t>
+        </is>
+      </c>
       <c r="X16" s="13" t="inlineStr">
         <is>
           <t>Kya tum meri madad karoge?</t>
@@ -4693,7 +4697,11 @@
           <t>Can I sit here?</t>
         </is>
       </c>
-      <c r="W20" s="13" t="inlineStr"/>
+      <c r="W20" s="14" t="inlineStr">
+        <is>
+          <t>Can I use your phone for a minute?</t>
+        </is>
+      </c>
       <c r="X20" s="13" t="inlineStr">
         <is>
           <t>Kya main andar aa sakta hoon?</t>
@@ -5545,7 +5553,11 @@
           <t>What do you call this in English?</t>
         </is>
       </c>
-      <c r="W24" s="13" t="inlineStr"/>
+      <c r="W24" s="14" t="inlineStr">
+        <is>
+          <t>What do you call "jhadu" in English?</t>
+        </is>
+      </c>
       <c r="X24" s="13" t="inlineStr">
         <is>
           <t>Chammach ko English mein kya kehte hain?</t>
@@ -7237,7 +7249,11 @@
           <t>I don't want to eat.</t>
         </is>
       </c>
-      <c r="W32" s="13" t="inlineStr"/>
+      <c r="W32" s="14" t="inlineStr">
+        <is>
+          <t>I don't want to be late for the train.</t>
+        </is>
+      </c>
       <c r="X32" s="13" t="inlineStr">
         <is>
           <t>Main aaj bahar nahi jaana chahta.</t>
@@ -7665,7 +7681,11 @@
           <t>My hobbies are reading and cooking.</t>
         </is>
       </c>
-      <c r="W34" s="13" t="inlineStr"/>
+      <c r="W34" s="14" t="inlineStr">
+        <is>
+          <t>My hobby is collecting old coins.</t>
+        </is>
+      </c>
       <c r="X34" s="13" t="inlineStr">
         <is>
           <t>Mera shauk painting karna hai.</t>
@@ -7869,7 +7889,11 @@
           <t>What's your number?</t>
         </is>
       </c>
-      <c r="W35" s="13" t="inlineStr"/>
+      <c r="W35" s="14" t="inlineStr">
+        <is>
+          <t>What's your favourite food?</t>
+        </is>
+      </c>
       <c r="X35" s="13" t="inlineStr">
         <is>
           <t>Tumhara naam kya hai?</t>
@@ -8285,7 +8309,11 @@
           <t>Which one do you like?</t>
         </is>
       </c>
-      <c r="W37" s="13" t="inlineStr"/>
+      <c r="W37" s="14" t="inlineStr">
+        <is>
+          <t>Which subject do you like the most?</t>
+        </is>
+      </c>
       <c r="X37" s="13" t="inlineStr">
         <is>
           <t>Tumhe kaunsa rang pasand hai?</t>
@@ -8697,7 +8725,11 @@
           <t>How many brothers do you have?</t>
         </is>
       </c>
-      <c r="W39" s="13" t="inlineStr"/>
+      <c r="W39" s="14" t="inlineStr">
+        <is>
+          <t>How many students do you have in your class?</t>
+        </is>
+      </c>
       <c r="X39" s="13" t="inlineStr">
         <is>
           <t>Tumhare paas kitni kitaabein hain?</t>
@@ -9325,7 +9357,11 @@
           <t>What did you do on the weekend?</t>
         </is>
       </c>
-      <c r="W42" s="13" t="inlineStr"/>
+      <c r="W42" s="14" t="inlineStr">
+        <is>
+          <t>What did you do last night?</t>
+        </is>
+      </c>
       <c r="X42" s="13" t="inlineStr">
         <is>
           <t>Tumne kal kya kiya?</t>
@@ -9529,7 +9565,11 @@
           <t>Where do you work?</t>
         </is>
       </c>
-      <c r="W43" s="13" t="inlineStr"/>
+      <c r="W43" s="14" t="inlineStr">
+        <is>
+          <t>Where do you buy your vegetables?</t>
+        </is>
+      </c>
       <c r="X43" s="13" t="inlineStr">
         <is>
           <t>Tum kahan rehte ho?</t>
@@ -9949,7 +9989,11 @@
           <t>Do you have change?</t>
         </is>
       </c>
-      <c r="W45" s="13" t="inlineStr"/>
+      <c r="W45" s="14" t="inlineStr">
+        <is>
+          <t>Do you have a charger I can use?</t>
+        </is>
+      </c>
       <c r="X45" s="13" t="inlineStr">
         <is>
           <t>Kya tumhare paas pen hai?</t>
@@ -12717,7 +12761,11 @@
           <t>The film is about to start.</t>
         </is>
       </c>
-      <c r="W58" s="13" t="inlineStr"/>
+      <c r="W58" s="14" t="inlineStr">
+        <is>
+          <t>Hurry up, the bus is about to leave.</t>
+        </is>
+      </c>
       <c r="X58" s="13" t="inlineStr">
         <is>
           <t>Main nikalne wala hoon.</t>
@@ -13569,7 +13617,11 @@
           <t>You should rest.</t>
         </is>
       </c>
-      <c r="W62" s="13" t="inlineStr"/>
+      <c r="W62" s="14" t="inlineStr">
+        <is>
+          <t>You should drink more water in summer.</t>
+        </is>
+      </c>
       <c r="X62" s="13" t="inlineStr">
         <is>
           <t>Tumhe doctor ko dikhana chahiye.</t>
@@ -14609,7 +14661,11 @@
           <t>She's the tallest in class.</t>
         </is>
       </c>
-      <c r="W67" s="13" t="inlineStr"/>
+      <c r="W67" s="14" t="inlineStr">
+        <is>
+          <t>Mount Everest is the highest mountain in the world.</t>
+        </is>
+      </c>
       <c r="X67" s="13" t="inlineStr">
         <is>
           <t>Yeh sabse achha phone hai.</t>
@@ -15025,7 +15081,11 @@
           <t>Either tea or coffee.</t>
         </is>
       </c>
-      <c r="W69" s="13" t="inlineStr"/>
+      <c r="W69" s="14" t="inlineStr">
+        <is>
+          <t>You can pay either by cash or by card.</t>
+        </is>
+      </c>
       <c r="X69" s="13" t="inlineStr">
         <is>
           <t>Ya toh aaj aao ya kal.</t>
@@ -15453,7 +15513,11 @@
           <t>Rice is grown in Punjab.</t>
         </is>
       </c>
-      <c r="W71" s="13" t="inlineStr"/>
+      <c r="W71" s="14" t="inlineStr">
+        <is>
+          <t>Tea is grown in Assam.</t>
+        </is>
+      </c>
       <c r="X71" s="13" t="inlineStr">
         <is>
           <t>Yahan English boli jaati hai.</t>
@@ -15653,7 +15717,11 @@
           <t>The Taj Mahal was built by Shah Jahan.</t>
         </is>
       </c>
-      <c r="W72" s="13" t="inlineStr"/>
+      <c r="W72" s="14" t="inlineStr">
+        <is>
+          <t>The bridge was opened in 2015.</t>
+        </is>
+      </c>
       <c r="X72" s="13" t="inlineStr">
         <is>
           <t>Yeh ghar 1990 mein banaya gaya tha.</t>
@@ -16473,7 +16541,11 @@
           <t>She asked me to help.</t>
         </is>
       </c>
-      <c r="W76" s="13" t="inlineStr"/>
+      <c r="W76" s="14" t="inlineStr">
+        <is>
+          <t>My teacher asked me to read the poem aloud.</t>
+        </is>
+      </c>
       <c r="X76" s="13" t="inlineStr">
         <is>
           <t>Usne mujhse wait karne ko kaha.</t>
@@ -16889,7 +16961,11 @@
           <t>I don't know what time it is.</t>
         </is>
       </c>
-      <c r="W78" s="13" t="inlineStr"/>
+      <c r="W78" s="14" t="inlineStr">
+        <is>
+          <t>I don't know what her phone number is.</t>
+        </is>
+      </c>
       <c r="X78" s="13" t="inlineStr">
         <is>
           <t>Mujhe nahi pata ki uska naam kya hai.</t>
@@ -17093,7 +17169,11 @@
           <t>I'm sure he's home.</t>
         </is>
       </c>
-      <c r="W79" s="13" t="inlineStr"/>
+      <c r="W79" s="14" t="inlineStr">
+        <is>
+          <t>I'm sure that the shop opens at ten.</t>
+        </is>
+      </c>
       <c r="X79" s="13" t="inlineStr">
         <is>
           <t>Mujhe yakeen hai ki tum pass ho jaoge.</t>
@@ -17305,7 +17385,11 @@
           <t>I don't think it's true.</t>
         </is>
       </c>
-      <c r="W80" s="13" t="inlineStr"/>
+      <c r="W80" s="14" t="inlineStr">
+        <is>
+          <t>I don't think we need an umbrella today.</t>
+        </is>
+      </c>
       <c r="X80" s="13" t="inlineStr">
         <is>
           <t>Mujhe nahi lagta ki woh aayega.</t>
@@ -17509,7 +17593,11 @@
           <t>I hope it doesn't rain.</t>
         </is>
       </c>
-      <c r="W81" s="13" t="inlineStr"/>
+      <c r="W81" s="14" t="inlineStr">
+        <is>
+          <t>I hope that you feel better soon.</t>
+        </is>
+      </c>
       <c r="X81" s="13" t="inlineStr">
         <is>
           <t>Mujhe ummeed hai ki tumhe job mil jaaye.</t>
@@ -17937,7 +18025,11 @@
           <t>She let me use her phone.</t>
         </is>
       </c>
-      <c r="W83" s="13" t="inlineStr"/>
+      <c r="W83" s="14" t="inlineStr">
+        <is>
+          <t>My brother let me ride his bike.</t>
+        </is>
+      </c>
       <c r="X83" s="13" t="inlineStr">
         <is>
           <t>Papa ne mujhe jaane diya.</t>
@@ -19393,7 +19485,11 @@
           <t>Should I take the job?</t>
         </is>
       </c>
-      <c r="W90" s="13" t="inlineStr"/>
+      <c r="W90" s="14" t="inlineStr">
+        <is>
+          <t>It's very cold. Should I wear a jacket?</t>
+        </is>
+      </c>
       <c r="X90" s="13" t="inlineStr">
         <is>
           <t>Kya mujhe usse call karna chahiye?</t>
@@ -19805,7 +19901,11 @@
           <t>I had to wait an hour.</t>
         </is>
       </c>
-      <c r="W92" s="13" t="inlineStr"/>
+      <c r="W92" s="14" t="inlineStr">
+        <is>
+          <t>The lift was broken, so I had to take the stairs.</t>
+        </is>
+      </c>
       <c r="X92" s="13" t="inlineStr">
         <is>
           <t>Mujhe paidal jaana pada.</t>
@@ -20649,7 +20749,11 @@
           <t>You must wear a helmet.</t>
         </is>
       </c>
-      <c r="W96" s="13" t="inlineStr"/>
+      <c r="W96" s="14" t="inlineStr">
+        <is>
+          <t>You must switch off your phone in the exam hall.</t>
+        </is>
+      </c>
       <c r="X96" s="13" t="inlineStr">
         <is>
           <t>Tum zaroor Goa jaana.</t>
@@ -21485,7 +21589,11 @@
           <t>I've finished eating.</t>
         </is>
       </c>
-      <c r="W100" s="13" t="inlineStr"/>
+      <c r="W100" s="14" t="inlineStr">
+        <is>
+          <t>I've finished reading the book you gave me.</t>
+        </is>
+      </c>
       <c r="X100" s="13" t="inlineStr">
         <is>
           <t>Maine packing khatam kar li.</t>
@@ -21689,7 +21797,11 @@
           <t>I forgot to call.</t>
         </is>
       </c>
-      <c r="W101" s="13" t="inlineStr"/>
+      <c r="W101" s="14" t="inlineStr">
+        <is>
+          <t>I forgot to bring my lunch today.</t>
+        </is>
+      </c>
       <c r="X101" s="13" t="inlineStr">
         <is>
           <t>Main darwaza lock karna bhool gaya.</t>
@@ -21897,7 +22009,11 @@
           <t>She's learning to swim.</t>
         </is>
       </c>
-      <c r="W102" s="13" t="inlineStr"/>
+      <c r="W102" s="14" t="inlineStr">
+        <is>
+          <t>My grandmother is learning to use WhatsApp.</t>
+        </is>
+      </c>
       <c r="X102" s="13" t="inlineStr">
         <is>
           <t>Main gaadi chalana seekh raha hoon.</t>
@@ -22105,7 +22221,11 @@
           <t>She started learning Hindi.</t>
         </is>
       </c>
-      <c r="W103" s="13" t="inlineStr"/>
+      <c r="W103" s="14" t="inlineStr">
+        <is>
+          <t>Last year I started learning the guitar.</t>
+        </is>
+      </c>
       <c r="X103" s="13" t="inlineStr">
         <is>
           <t>Maine gym jaana shuru kiya.</t>
@@ -23149,7 +23269,11 @@
           <t>I'm scared to fly.</t>
         </is>
       </c>
-      <c r="W108" s="13" t="inlineStr"/>
+      <c r="W108" s="14" t="inlineStr">
+        <is>
+          <t>I'm scared to swim in the deep end.</t>
+        </is>
+      </c>
       <c r="X108" s="13" t="inlineStr">
         <is>
           <t>Main stage par bolne se darta hoon.</t>
@@ -23573,7 +23697,11 @@
           <t>I'm glad to help.</t>
         </is>
       </c>
-      <c r="W110" s="13" t="inlineStr"/>
+      <c r="W110" s="14" t="inlineStr">
+        <is>
+          <t>I'm glad to see you again.</t>
+        </is>
+      </c>
       <c r="X110" s="13" t="inlineStr">
         <is>
           <t>Mujhe yeh sunkar khushi hui.</t>
@@ -24417,7 +24545,11 @@
           <t>How do you cook dal?</t>
         </is>
       </c>
-      <c r="W114" s="13" t="inlineStr"/>
+      <c r="W114" s="14" t="inlineStr">
+        <is>
+          <t>How do you remember new words?</t>
+        </is>
+      </c>
       <c r="X114" s="13" t="inlineStr">
         <is>
           <t>Tum English kaise practise karte ho?</t>
@@ -24833,7 +24965,11 @@
           <t>Why are you crying?</t>
         </is>
       </c>
-      <c r="W116" s="13" t="inlineStr"/>
+      <c r="W116" s="14" t="inlineStr">
+        <is>
+          <t>Why are you running? We have time.</t>
+        </is>
+      </c>
       <c r="X116" s="13" t="inlineStr">
         <is>
           <t>Tum has kyon rahe ho?</t>
@@ -25253,7 +25389,11 @@
           <t>Why do you like this song?</t>
         </is>
       </c>
-      <c r="W118" s="13" t="inlineStr"/>
+      <c r="W118" s="14" t="inlineStr">
+        <is>
+          <t>Why do you like living in a small town?</t>
+        </is>
+      </c>
       <c r="X118" s="13" t="inlineStr">
         <is>
           <t>Tumhe cricket kyon pasand hai?</t>
@@ -25457,7 +25597,11 @@
           <t>Do you think he's right?</t>
         </is>
       </c>
-      <c r="W119" s="13" t="inlineStr"/>
+      <c r="W119" s="14" t="inlineStr">
+        <is>
+          <t>Do you think we'll get tickets for the match?</t>
+        </is>
+      </c>
       <c r="X119" s="13" t="inlineStr">
         <is>
           <t>Tumhe kya lagta hai, baarish hogi?</t>
@@ -25665,7 +25809,11 @@
           <t>Which is better, this or that?</t>
         </is>
       </c>
-      <c r="W120" s="13" t="inlineStr"/>
+      <c r="W120" s="14" t="inlineStr">
+        <is>
+          <t>Which is better, the train or the bus to Jaipur?</t>
+        </is>
+      </c>
       <c r="X120" s="13" t="inlineStr">
         <is>
           <t>Kaunsa behtar hai, chai ya coffee?</t>
@@ -25873,7 +26021,11 @@
           <t>Which school is the best?</t>
         </is>
       </c>
-      <c r="W121" s="13" t="inlineStr"/>
+      <c r="W121" s="14" t="inlineStr">
+        <is>
+          <t>Which app is the best for learning English?</t>
+        </is>
+      </c>
       <c r="X121" s="13" t="inlineStr">
         <is>
           <t>Kaunsa phone sabse achha hai?</t>
@@ -26085,7 +26237,11 @@
           <t>I haven't finished yet.</t>
         </is>
       </c>
-      <c r="W122" s="13" t="inlineStr"/>
+      <c r="W122" s="14" t="inlineStr">
+        <is>
+          <t>I haven't paid the electricity bill yet.</t>
+        </is>
+      </c>
       <c r="X122" s="13" t="inlineStr">
         <is>
           <t>Maine abhi tak khana nahi khaya.</t>
@@ -26497,7 +26653,11 @@
           <t>Were you working at 6?</t>
         </is>
       </c>
-      <c r="W124" s="13" t="inlineStr"/>
+      <c r="W124" s="14" t="inlineStr">
+        <is>
+          <t>Were you watching TV when I called?</t>
+        </is>
+      </c>
       <c r="X124" s="13" t="inlineStr">
         <is>
           <t>Kya tum so rahe the?</t>
@@ -27333,7 +27493,11 @@
           <t>Whenever it rains, I stay in.</t>
         </is>
       </c>
-      <c r="W128" s="13" t="inlineStr"/>
+      <c r="W128" s="14" t="inlineStr">
+        <is>
+          <t>Whenever I visit my grandmother, she makes halwa.</t>
+        </is>
+      </c>
       <c r="X128" s="13" t="inlineStr">
         <is>
           <t>Jab bhi main usse milta hoon, woh muskurata hai.</t>
@@ -28385,7 +28549,11 @@
           <t>It's time to go.</t>
         </is>
       </c>
-      <c r="W133" s="13" t="inlineStr"/>
+      <c r="W133" s="14" t="inlineStr">
+        <is>
+          <t>It's time to start the class.</t>
+        </is>
+      </c>
       <c r="X133" s="13" t="inlineStr">
         <is>
           <t>Sone ka time ho gaya hai.</t>
@@ -29017,7 +29185,11 @@
           <t>There's no need to shout.</t>
         </is>
       </c>
-      <c r="W136" s="13" t="inlineStr"/>
+      <c r="W136" s="14" t="inlineStr">
+        <is>
+          <t>There's no need to bring food; lunch is provided.</t>
+        </is>
+      </c>
       <c r="X136" s="13" t="inlineStr">
         <is>
           <t>Chinta karne ki koi zaroorat nahi.</t>
@@ -29225,7 +29397,11 @@
           <t>It's good that it stopped raining.</t>
         </is>
       </c>
-      <c r="W137" s="13" t="inlineStr"/>
+      <c r="W137" s="14" t="inlineStr">
+        <is>
+          <t>It's good that you told me the truth.</t>
+        </is>
+      </c>
       <c r="X137" s="13" t="inlineStr">
         <is>
           <t>Yeh achha hai ki tum aa gaye.</t>
@@ -30069,7 +30245,11 @@
           <t>She likes both dogs and cats.</t>
         </is>
       </c>
-      <c r="W141" s="13" t="inlineStr"/>
+      <c r="W141" s="14" t="inlineStr">
+        <is>
+          <t>I like both Hindi and English films.</t>
+        </is>
+      </c>
       <c r="X141" s="13" t="inlineStr">
         <is>
           <t>Mujhe chai aur coffee dono pasand hain.</t>
@@ -30277,7 +30457,11 @@
           <t>Come as soon as possible.</t>
         </is>
       </c>
-      <c r="W142" s="13" t="inlineStr"/>
+      <c r="W142" s="14" t="inlineStr">
+        <is>
+          <t>Please reply as soon as possible.</t>
+        </is>
+      </c>
       <c r="X142" s="13" t="inlineStr">
         <is>
           <t>Jitna ho sake utna practice karo.</t>
@@ -31997,7 +32181,11 @@
           <t>I keep losing my keys.</t>
         </is>
       </c>
-      <c r="W150" s="13" t="inlineStr"/>
+      <c r="W150" s="14" t="inlineStr">
+        <is>
+          <t>My little brother keeps asking for chocolate.</t>
+        </is>
+      </c>
       <c r="X150" s="13" t="inlineStr">
         <is>
           <t>Main naam bhoolta rehta hoon.</t>
@@ -32409,7 +32597,11 @@
           <t>The film had started before we came.</t>
         </is>
       </c>
-      <c r="W152" s="13" t="inlineStr"/>
+      <c r="W152" s="14" t="inlineStr">
+        <is>
+          <t>The shop had already closed before I arrived.</t>
+        </is>
+      </c>
       <c r="X152" s="13" t="inlineStr">
         <is>
           <t>Mere pahunchne se pehle hi train ja chuki thi.</t>
@@ -32621,7 +32813,11 @@
           <t>I'm thinking of buying a car.</t>
         </is>
       </c>
-      <c r="W153" s="13" t="inlineStr"/>
+      <c r="W153" s="14" t="inlineStr">
+        <is>
+          <t>I'm thinking of joining a dance class.</t>
+        </is>
+      </c>
       <c r="X153" s="13" t="inlineStr">
         <is>
           <t>Main MBA karne ka soch raha hoon.</t>
@@ -33869,7 +34065,11 @@
           <t>How long have you been waiting?</t>
         </is>
       </c>
-      <c r="W159" s="13" t="inlineStr"/>
+      <c r="W159" s="14" t="inlineStr">
+        <is>
+          <t>How long have you been living in Hyderabad?</t>
+        </is>
+      </c>
       <c r="X159" s="13" t="inlineStr">
         <is>
           <t>Tum kab se English seekh rahe ho?</t>
@@ -34697,7 +34897,11 @@
           <t>He's neither rich nor poor.</t>
         </is>
       </c>
-      <c r="W163" s="13" t="inlineStr"/>
+      <c r="W163" s="14" t="inlineStr">
+        <is>
+          <t>The room was neither clean nor quiet.</t>
+        </is>
+      </c>
       <c r="X163" s="13" t="inlineStr">
         <is>
           <t>Mujhe na chai pasand hai na coffee.</t>
@@ -34897,7 +35101,11 @@
           <t>The work will be done by Friday.</t>
         </is>
       </c>
-      <c r="W164" s="13" t="inlineStr"/>
+      <c r="W164" s="14" t="inlineStr">
+        <is>
+          <t>The new road will be opened next month.</t>
+        </is>
+      </c>
       <c r="X164" s="13" t="inlineStr">
         <is>
           <t>Result kal ghoshit kiya jaayega.</t>
@@ -35101,7 +35309,11 @@
           <t>The room has been cleaned.</t>
         </is>
       </c>
-      <c r="W165" s="13" t="inlineStr"/>
+      <c r="W165" s="14" t="inlineStr">
+        <is>
+          <t>The bill has been paid.</t>
+        </is>
+      </c>
       <c r="X165" s="13" t="inlineStr">
         <is>
           <t>Aapka order bhej diya gaya hai.</t>
@@ -35713,7 +35925,11 @@
           <t>Waste should be recycled.</t>
         </is>
       </c>
-      <c r="W168" s="13" t="inlineStr"/>
+      <c r="W168" s="14" t="inlineStr">
+        <is>
+          <t>Old phones should be recycled, not thrown away.</t>
+        </is>
+      </c>
       <c r="X168" s="13" t="inlineStr">
         <is>
           <t>Is niyam ko badla jaana chahiye.</t>
@@ -36121,7 +36337,11 @@
           <t>I was given a chance.</t>
         </is>
       </c>
-      <c r="W170" s="13" t="inlineStr"/>
+      <c r="W170" s="14" t="inlineStr">
+        <is>
+          <t>I was given a gift by my students.</t>
+        </is>
+      </c>
       <c r="X170" s="13" t="inlineStr">
         <is>
           <t>Mujhe ek certificate diya gaya.</t>
@@ -36537,7 +36757,11 @@
           <t>Mum told me not to worry.</t>
         </is>
       </c>
-      <c r="W172" s="13" t="inlineStr"/>
+      <c r="W172" s="14" t="inlineStr">
+        <is>
+          <t>The doctor told me not to eat fried food.</t>
+        </is>
+      </c>
       <c r="X172" s="13" t="inlineStr">
         <is>
           <t>Usne mujhse late na aane ko kaha.</t>
@@ -36741,7 +36965,11 @@
           <t>She asked if we were coming.</t>
         </is>
       </c>
-      <c r="W173" s="13" t="inlineStr"/>
+      <c r="W173" s="14" t="inlineStr">
+        <is>
+          <t>The teacher asked if we had any questions.</t>
+        </is>
+      </c>
       <c r="X173" s="13" t="inlineStr">
         <is>
           <t>Usne poocha ki kya main free hoon.</t>
@@ -36945,7 +37173,11 @@
           <t>She asked where I lived.</t>
         </is>
       </c>
-      <c r="W174" s="13" t="inlineStr"/>
+      <c r="W174" s="14" t="inlineStr">
+        <is>
+          <t>A tourist asked me where the museum was.</t>
+        </is>
+      </c>
       <c r="X174" s="13" t="inlineStr">
         <is>
           <t>Usne poocha ki station kahan hai.</t>
@@ -37777,7 +38009,11 @@
           <t>Could you tell me where the lift is?</t>
         </is>
       </c>
-      <c r="W178" s="13" t="inlineStr"/>
+      <c r="W178" s="14" t="inlineStr">
+        <is>
+          <t>Could you tell me how much this costs?</t>
+        </is>
+      </c>
       <c r="X178" s="13" t="inlineStr">
         <is>
           <t>Kya aap bata sakte hain ki bank kab khulta hai?</t>
@@ -37977,7 +38213,11 @@
           <t>What I need is a good job.</t>
         </is>
       </c>
-      <c r="W179" s="13" t="inlineStr"/>
+      <c r="W179" s="14" t="inlineStr">
+        <is>
+          <t>What I need is a cup of hot tea.</t>
+        </is>
+      </c>
       <c r="X179" s="13" t="inlineStr">
         <is>
           <t>Mujhe jo chahiye woh hai thoda aaraam.</t>
@@ -38609,7 +38849,11 @@
           <t>She advised me to wait.</t>
         </is>
       </c>
-      <c r="W182" s="13" t="inlineStr"/>
+      <c r="W182" s="14" t="inlineStr">
+        <is>
+          <t>My teacher advised me to read English newspapers.</t>
+        </is>
+      </c>
       <c r="X182" s="13" t="inlineStr">
         <is>
           <t>Doctor ne mujhe aaraam karne ki salah di.</t>
@@ -39017,7 +39261,11 @@
           <t>I got my hair cut.</t>
         </is>
       </c>
-      <c r="W184" s="13" t="inlineStr"/>
+      <c r="W184" s="14" t="inlineStr">
+        <is>
+          <t>I got my watch fixed at the market.</t>
+        </is>
+      </c>
       <c r="X184" s="13" t="inlineStr">
         <is>
           <t>Maine apna phone theek karwaya.</t>
@@ -39217,7 +39465,11 @@
           <t>I have my car washed weekly.</t>
         </is>
       </c>
-      <c r="W185" s="13" t="inlineStr"/>
+      <c r="W185" s="14" t="inlineStr">
+        <is>
+          <t>We have our house painted every five years.</t>
+        </is>
+      </c>
       <c r="X185" s="13" t="inlineStr">
         <is>
           <t>Main har mahine baal katwata hoon.</t>
@@ -39417,7 +39669,11 @@
           <t>Dad allowed me to go.</t>
         </is>
       </c>
-      <c r="W186" s="13" t="inlineStr"/>
+      <c r="W186" s="14" t="inlineStr">
+        <is>
+          <t>The guard allowed me to park near the gate.</t>
+        </is>
+      </c>
       <c r="X186" s="13" t="inlineStr">
         <is>
           <t>Boss ne mujhe ghar se kaam karne ki ijazat di.</t>
@@ -39833,7 +40089,11 @@
           <t>She must be at home.</t>
         </is>
       </c>
-      <c r="W188" s="13" t="inlineStr"/>
+      <c r="W188" s="14" t="inlineStr">
+        <is>
+          <t>You walked ten kilometres? You must be hungry.</t>
+        </is>
+      </c>
       <c r="X188" s="13" t="inlineStr">
         <is>
           <t>Woh zaroor thaka hoga.</t>
@@ -40245,7 +40505,11 @@
           <t>That can't be true.</t>
         </is>
       </c>
-      <c r="W190" s="13" t="inlineStr"/>
+      <c r="W190" s="14" t="inlineStr">
+        <is>
+          <t>He just ate two plates of rice. He can't be hungry.</t>
+        </is>
+      </c>
       <c r="X190" s="13" t="inlineStr">
         <is>
           <t>Woh abhi office mein nahi ho sakta.</t>
@@ -40449,7 +40713,11 @@
           <t>She must have forgotten.</t>
         </is>
       </c>
-      <c r="W191" s="13" t="inlineStr"/>
+      <c r="W191" s="14" t="inlineStr">
+        <is>
+          <t>The ground is wet. It must have rained last night.</t>
+        </is>
+      </c>
       <c r="X191" s="13" t="inlineStr">
         <is>
           <t>Usne zaroor train miss kar di hogi.</t>
@@ -40657,7 +40925,11 @@
           <t>She might have left.</t>
         </is>
       </c>
-      <c r="W192" s="13" t="inlineStr"/>
+      <c r="W192" s="14" t="inlineStr">
+        <is>
+          <t>I can't find my keys. I might have left them at work.</t>
+        </is>
+      </c>
       <c r="X192" s="13" t="inlineStr">
         <is>
           <t>Shayad woh bhool gaya ho.</t>
@@ -40865,7 +41137,11 @@
           <t>She can't have forgotten.</t>
         </is>
       </c>
-      <c r="W193" s="13" t="inlineStr"/>
+      <c r="W193" s="14" t="inlineStr">
+        <is>
+          <t>She can't have finished the book already; it's 500 pages.</t>
+        </is>
+      </c>
       <c r="X193" s="13" t="inlineStr">
         <is>
           <t>Usne yeh akele nahi kiya hoga.</t>
@@ -41069,7 +41345,11 @@
           <t>You could have told me.</t>
         </is>
       </c>
-      <c r="W194" s="13" t="inlineStr"/>
+      <c r="W194" s="14" t="inlineStr">
+        <is>
+          <t>I could have taken the earlier bus, but I missed it.</t>
+        </is>
+      </c>
       <c r="X194" s="13" t="inlineStr">
         <is>
           <t>Main jeet sakta tha.</t>
@@ -41481,7 +41761,11 @@
           <t>I shouldn't have shouted.</t>
         </is>
       </c>
-      <c r="W196" s="13" t="inlineStr"/>
+      <c r="W196" s="14" t="inlineStr">
+        <is>
+          <t>I shouldn't have stayed up so late.</t>
+        </is>
+      </c>
       <c r="X196" s="13" t="inlineStr">
         <is>
           <t>Mujhe itna nahi khana chahiye tha.</t>
@@ -41693,7 +41977,11 @@
           <t>You'd better study.</t>
         </is>
       </c>
-      <c r="W197" s="13" t="inlineStr"/>
+      <c r="W197" s="14" t="inlineStr">
+        <is>
+          <t>It's getting dark. You'd better go home.</t>
+        </is>
+      </c>
       <c r="X197" s="13" t="inlineStr">
         <is>
           <t>Behtar hoga ki tum abhi nikal jao.</t>
@@ -42105,7 +42393,11 @@
           <t>You didn't need to wait.</t>
         </is>
       </c>
-      <c r="W199" s="13" t="inlineStr"/>
+      <c r="W199" s="14" t="inlineStr">
+        <is>
+          <t>You didn't need to pick me up; I could take an auto.</t>
+        </is>
+      </c>
       <c r="X199" s="13" t="inlineStr">
         <is>
           <t>Tumhe gift laane ki zaroorat nahi thi.</t>
@@ -42313,7 +42605,11 @@
           <t>It might not rain.</t>
         </is>
       </c>
-      <c r="W200" s="13" t="inlineStr"/>
+      <c r="W200" s="14" t="inlineStr">
+        <is>
+          <t>Take the umbrella. The rain might not stop soon.</t>
+        </is>
+      </c>
       <c r="X200" s="13" t="inlineStr">
         <is>
           <t>Ho sakta hai ki woh na aaye.</t>
@@ -42521,7 +42817,11 @@
           <t>The parcel should come by Friday.</t>
         </is>
       </c>
-      <c r="W201" s="13" t="inlineStr"/>
+      <c r="W201" s="14" t="inlineStr">
+        <is>
+          <t>The results should be online by Monday.</t>
+        </is>
+      </c>
       <c r="X201" s="13" t="inlineStr">
         <is>
           <t>Train ko paanch baje tak aa jaana chahiye.</t>
@@ -42721,7 +43021,11 @@
           <t>We had no choice but to wait.</t>
         </is>
       </c>
-      <c r="W202" s="13" t="inlineStr"/>
+      <c r="W202" s="14" t="inlineStr">
+        <is>
+          <t>The bus didn't come, so I had no choice but to walk.</t>
+        </is>
+      </c>
       <c r="X202" s="13" t="inlineStr">
         <is>
           <t>Mujhe maafi maangni hi padegi.</t>
@@ -43345,7 +43649,11 @@
           <t>She promised to help.</t>
         </is>
       </c>
-      <c r="W205" s="13" t="inlineStr"/>
+      <c r="W205" s="14" t="inlineStr">
+        <is>
+          <t>I promised to visit my grandparents this summer.</t>
+        </is>
+      </c>
       <c r="X205" s="13" t="inlineStr">
         <is>
           <t>Maine usse call karne ka waada kiya.</t>
@@ -43553,7 +43861,11 @@
           <t>She refused to answer.</t>
         </is>
       </c>
-      <c r="W206" s="13" t="inlineStr"/>
+      <c r="W206" s="14" t="inlineStr">
+        <is>
+          <t>The shopkeeper refused to give me a refund.</t>
+        </is>
+      </c>
       <c r="X206" s="13" t="inlineStr">
         <is>
           <t>Usne paise lene se mana kar diya.</t>
@@ -43969,7 +44281,11 @@
           <t>I find it hard to focus.</t>
         </is>
       </c>
-      <c r="W208" s="13" t="inlineStr"/>
+      <c r="W208" s="14" t="inlineStr">
+        <is>
+          <t>I find it hard to speak English in front of many people.</t>
+        </is>
+      </c>
       <c r="X208" s="13" t="inlineStr">
         <is>
           <t>Mujhe subah jaldi uthne mein mushkil hoti hai.</t>
@@ -44173,7 +44489,11 @@
           <t>I got a chance to meet her.</t>
         </is>
       </c>
-      <c r="W209" s="13" t="inlineStr"/>
+      <c r="W209" s="14" t="inlineStr">
+        <is>
+          <t>At the festival, I got a chance to meet a famous singer.</t>
+        </is>
+      </c>
       <c r="X209" s="13" t="inlineStr">
         <is>
           <t>Mujhe London jaane ka mauka mila.</t>
@@ -44385,7 +44705,11 @@
           <t>I don't mind helping.</t>
         </is>
       </c>
-      <c r="W210" s="13" t="inlineStr"/>
+      <c r="W210" s="14" t="inlineStr">
+        <is>
+          <t>I don't mind sitting at the back.</t>
+        </is>
+      </c>
       <c r="X210" s="13" t="inlineStr">
         <is>
           <t>Mujhe wait karne mein koi dikkat nahi.</t>
@@ -44589,7 +44913,11 @@
           <t>Try adding more salt.</t>
         </is>
       </c>
-      <c r="W211" s="13" t="inlineStr"/>
+      <c r="W211" s="14" t="inlineStr">
+        <is>
+          <t>I tried calling her, but she didn't pick up.</t>
+        </is>
+      </c>
       <c r="X211" s="13" t="inlineStr">
         <is>
           <t>Maine phone restart karke dekha.</t>
@@ -44789,7 +45117,11 @@
           <t>I regret not studying.</t>
         </is>
       </c>
-      <c r="W212" s="13" t="inlineStr"/>
+      <c r="W212" s="14" t="inlineStr">
+        <is>
+          <t>I regret not learning to swim as a child.</t>
+        </is>
+      </c>
       <c r="X212" s="13" t="inlineStr">
         <is>
           <t>Mujhe usse jhooth bolne ka pachhtava hai.</t>
@@ -44997,7 +45329,11 @@
           <t>She's determined to win.</t>
         </is>
       </c>
-      <c r="W213" s="13" t="inlineStr"/>
+      <c r="W213" s="14" t="inlineStr">
+        <is>
+          <t>After failing once, he's determined to pass this time.</t>
+        </is>
+      </c>
       <c r="X213" s="13" t="inlineStr">
         <is>
           <t>Maine English seekhne ki thaan li hai.</t>
@@ -45421,7 +45757,11 @@
           <t>I'll give up eating sugar.</t>
         </is>
       </c>
-      <c r="W215" s="13" t="inlineStr"/>
+      <c r="W215" s="14" t="inlineStr">
+        <is>
+          <t>For my health, I'll give up drinking cold drinks.</t>
+        </is>
+      </c>
       <c r="X215" s="13" t="inlineStr">
         <is>
           <t>Main smoking chhod dunga.</t>
@@ -45625,7 +45965,11 @@
           <t>I suggest trying this.</t>
         </is>
       </c>
-      <c r="W216" s="13" t="inlineStr"/>
+      <c r="W216" s="14" t="inlineStr">
+        <is>
+          <t>I suggest taking the metro; it's faster.</t>
+        </is>
+      </c>
       <c r="X216" s="13" t="inlineStr">
         <is>
           <t>Main suggest karta hoon ki hum jaldi niklein.</t>
@@ -46041,7 +46385,11 @@
           <t>I spent the day cooking.</t>
         </is>
       </c>
-      <c r="W218" s="13" t="inlineStr"/>
+      <c r="W218" s="14" t="inlineStr">
+        <is>
+          <t>We spent the whole evening talking about old times.</t>
+        </is>
+      </c>
       <c r="X218" s="13" t="inlineStr">
         <is>
           <t>Maine yeh seekhne mein teen ghante bitaye.</t>
@@ -46245,7 +46593,11 @@
           <t>I had trouble sleeping.</t>
         </is>
       </c>
-      <c r="W219" s="13" t="inlineStr"/>
+      <c r="W219" s="14" t="inlineStr">
+        <is>
+          <t>I had trouble understanding his accent.</t>
+        </is>
+      </c>
       <c r="X219" s="13" t="inlineStr">
         <is>
           <t>Mujhe ghar dhoondhne mein dikkat hui.</t>
@@ -46449,7 +46801,11 @@
           <t>I couldn't help crying.</t>
         </is>
       </c>
-      <c r="W220" s="13" t="inlineStr"/>
+      <c r="W220" s="14" t="inlineStr">
+        <is>
+          <t>The film was so sad that I couldn't help crying.</t>
+        </is>
+      </c>
       <c r="X220" s="13" t="inlineStr">
         <is>
           <t>Main hasne se khud ko rok nahi paaya.</t>
@@ -46653,7 +47009,11 @@
           <t>Who broke the glass?</t>
         </is>
       </c>
-      <c r="W221" s="13" t="inlineStr"/>
+      <c r="W221" s="14" t="inlineStr">
+        <is>
+          <t>Who left the tap open?</t>
+        </is>
+      </c>
       <c r="X221" s="13" t="inlineStr">
         <is>
           <t>Yeh kisne banaya?</t>
@@ -46853,7 +47213,11 @@
           <t>What's the best way to get there?</t>
         </is>
       </c>
-      <c r="W222" s="13" t="inlineStr"/>
+      <c r="W222" s="14" t="inlineStr">
+        <is>
+          <t>What's the best way to save money?</t>
+        </is>
+      </c>
       <c r="X222" s="13" t="inlineStr">
         <is>
           <t>English seekhne ka sabse achha tareeka kya hai?</t>
@@ -47065,7 +47429,11 @@
           <t>What made you choose this city?</t>
         </is>
       </c>
-      <c r="W223" s="13" t="inlineStr"/>
+      <c r="W223" s="14" t="inlineStr">
+        <is>
+          <t>What made you choose this college?</t>
+        </is>
+      </c>
       <c r="X223" s="13" t="inlineStr">
         <is>
           <t>Tumne teaching kyon chuni?</t>
@@ -47265,7 +47633,11 @@
           <t>I haven't eaten for hours.</t>
         </is>
       </c>
-      <c r="W224" s="13" t="inlineStr"/>
+      <c r="W224" s="14" t="inlineStr">
+        <is>
+          <t>I haven't seen my cousins for a long time.</t>
+        </is>
+      </c>
       <c r="X224" s="13" t="inlineStr">
         <is>
           <t>Maine do din se usse baat nahi ki.</t>
@@ -47469,7 +47841,11 @@
           <t>It's been ages since I cooked.</t>
         </is>
       </c>
-      <c r="W225" s="13" t="inlineStr"/>
+      <c r="W225" s="14" t="inlineStr">
+        <is>
+          <t>It's been two years since I visited my village.</t>
+        </is>
+      </c>
       <c r="X225" s="13" t="inlineStr">
         <is>
           <t>Usse mile hue ek saal ho gaya.</t>
@@ -47673,7 +48049,11 @@
           <t>I was going to cook, but I was tired.</t>
         </is>
       </c>
-      <c r="W226" s="13" t="inlineStr"/>
+      <c r="W226" s="14" t="inlineStr">
+        <is>
+          <t>I was going to buy the shoes, but they were too costly.</t>
+        </is>
+      </c>
       <c r="X226" s="13" t="inlineStr">
         <is>
           <t>Main call karne wala tha, lekin bhool gaya.</t>
@@ -47881,7 +48261,11 @@
           <t>She had never seen snow before.</t>
         </is>
       </c>
-      <c r="W227" s="13" t="inlineStr"/>
+      <c r="W227" s="14" t="inlineStr">
+        <is>
+          <t>I had never eaten sushi before that day.</t>
+        </is>
+      </c>
       <c r="X227" s="13" t="inlineStr">
         <is>
           <t>Maine pehle kabhi hawai jahaz mein safar nahi kiya tha.</t>
@@ -48293,7 +48677,11 @@
           <t>She's always losing her keys.</t>
         </is>
       </c>
-      <c r="W229" s="13" t="inlineStr"/>
+      <c r="W229" s="14" t="inlineStr">
+        <is>
+          <t>My neighbour is always playing loud music.</t>
+        </is>
+      </c>
       <c r="X229" s="13" t="inlineStr">
         <is>
           <t>Woh hamesha shikayat karta rehta hai.</t>
@@ -48497,7 +48885,11 @@
           <t>She didn't use to like maths.</t>
         </is>
       </c>
-      <c r="W230" s="13" t="inlineStr"/>
+      <c r="W230" s="14" t="inlineStr">
+        <is>
+          <t>I didn't use to like vegetables, but now I do.</t>
+        </is>
+      </c>
       <c r="X230" s="13" t="inlineStr">
         <is>
           <t>Main pehle chai nahi peeta tha.</t>
@@ -48697,7 +49089,11 @@
           <t>She had been working there for years when she left.</t>
         </is>
       </c>
-      <c r="W231" s="13" t="inlineStr"/>
+      <c r="W231" s="14" t="inlineStr">
+        <is>
+          <t>We had been walking for two hours when it started to rain.</t>
+        </is>
+      </c>
       <c r="X231" s="13" t="inlineStr">
         <is>
           <t>Main ek ghante se wait kar raha tha, tab woh aaya.</t>
@@ -49105,7 +49501,11 @@
           <t>If you had called, I would have come.</t>
         </is>
       </c>
-      <c r="W233" s="13" t="inlineStr"/>
+      <c r="W233" s="14" t="inlineStr">
+        <is>
+          <t>If I had left earlier, I would have caught the train.</t>
+        </is>
+      </c>
       <c r="X233" s="13" t="inlineStr">
         <is>
           <t>Agar maine padhai ki hoti, toh main pass ho jaata.</t>
@@ -49305,7 +49705,11 @@
           <t>You can go, as long as you're back by 9.</t>
         </is>
       </c>
-      <c r="W234" s="13" t="inlineStr"/>
+      <c r="W234" s="14" t="inlineStr">
+        <is>
+          <t>As long as you're honest, I'll help you.</t>
+        </is>
+      </c>
       <c r="X234" s="13" t="inlineStr">
         <is>
           <t>Jab tak tum mehnat karoge, tum safal hoge.</t>
@@ -49729,7 +50133,11 @@
           <t>Save the file in case it crashes.</t>
         </is>
       </c>
-      <c r="W236" s="13" t="inlineStr"/>
+      <c r="W236" s="14" t="inlineStr">
+        <is>
+          <t>Keep some water in the car in case you get thirsty.</t>
+        </is>
+      </c>
       <c r="X236" s="13" t="inlineStr">
         <is>
           <t>Chhata le lo, kahin baarish na ho jaaye.</t>
@@ -49929,7 +50337,11 @@
           <t>Even if you shout, I won't go.</t>
         </is>
       </c>
-      <c r="W237" s="13" t="inlineStr"/>
+      <c r="W237" s="14" t="inlineStr">
+        <is>
+          <t>Even if he says sorry, I won't forget it.</t>
+        </is>
+      </c>
       <c r="X237" s="13" t="inlineStr">
         <is>
           <t>Chahe baarish ho, main phir bhi aaunga.</t>
@@ -50137,7 +50549,11 @@
           <t>I wish I could come.</t>
         </is>
       </c>
-      <c r="W238" s="13" t="inlineStr"/>
+      <c r="W238" s="14" t="inlineStr">
+        <is>
+          <t>I wish I could visit my family more often.</t>
+        </is>
+      </c>
       <c r="X238" s="13" t="inlineStr">
         <is>
           <t>Kaash main French bol pata.</t>
@@ -50337,7 +50753,11 @@
           <t>I wish I had listened.</t>
         </is>
       </c>
-      <c r="W239" s="13" t="inlineStr"/>
+      <c r="W239" s="14" t="inlineStr">
+        <is>
+          <t>I wish I had brought a jacket; it's so cold.</t>
+        </is>
+      </c>
       <c r="X239" s="13" t="inlineStr">
         <is>
           <t>Kaash maine pehle shuru kiya hota.</t>
@@ -50757,7 +51177,11 @@
           <t>Suppose it rained, what would we do?</t>
         </is>
       </c>
-      <c r="W241" s="13" t="inlineStr"/>
+      <c r="W241" s="14" t="inlineStr">
+        <is>
+          <t>Suppose you lost your phone, what would you do?</t>
+        </is>
+      </c>
       <c r="X241" s="13" t="inlineStr">
         <is>
           <t>Maan lo ki tumhari lottery lag jaaye, toh kya karoge?</t>
@@ -51181,7 +51605,11 @@
           <t>It's worth trying.</t>
         </is>
       </c>
-      <c r="W243" s="13" t="inlineStr"/>
+      <c r="W243" s="14" t="inlineStr">
+        <is>
+          <t>Ooty is worth visiting in summer.</t>
+        </is>
+      </c>
       <c r="X243" s="13" t="inlineStr">
         <is>
           <t>Yeh film dekhne layak hai.</t>
@@ -51593,7 +52021,11 @@
           <t>It doesn't matter if you're late.</t>
         </is>
       </c>
-      <c r="W245" s="13" t="inlineStr"/>
+      <c r="W245" s="14" t="inlineStr">
+        <is>
+          <t>It doesn't matter what you wear; just come.</t>
+        </is>
+      </c>
       <c r="X245" s="13" t="inlineStr">
         <is>
           <t>Koi fark nahi padta ki tum kahan se ho.</t>
@@ -52013,7 +52445,11 @@
           <t>She's such a kind person that everyone likes her.</t>
         </is>
       </c>
-      <c r="W247" s="13" t="inlineStr"/>
+      <c r="W247" s="14" t="inlineStr">
+        <is>
+          <t>It was such a hot day that we stayed indoors.</t>
+        </is>
+      </c>
       <c r="X247" s="13" t="inlineStr">
         <is>
           <t>Woh itni achhi film thi ki maine do baar dekhi.</t>

</xml_diff>